<commit_message>
Atualiza dados de certificados (Dia/Mes/Ano + carga horaria) e inclui carga horaria no certificado e e-mail
</commit_message>
<xml_diff>
--- a/assets/Modelo Certificado.xlsx
+++ b/assets/Modelo Certificado.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30408"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://atlheticanutrition-my.sharepoint.com/personal/digital_platforms_nutramerica_com_br/Documents/DEV/TOTEN CERTIFICADO/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="36" documentId="8_{42677D5F-0A19-4617-994D-499172CF4C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{CFD6CECD-0153-45FA-A873-EDD3C5D75362}"/>
+  <xr:revisionPtr revIDLastSave="66" documentId="8_{42677D5F-0A19-4617-994D-499172CF4C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39226497-9F1D-4A34-A42C-E5A2AB1BE553}"/>
   <bookViews>
-    <workbookView xWindow="8420" yWindow="3840" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="8150" yWindow="2570" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Planilha Modelo" sheetId="1" r:id="rId1"/>
@@ -27,16 +27,17 @@
         <xcalcf:feature name="microsoft.com:FV"/>
         <xcalcf:feature name="microsoft.com:CNMTM"/>
         <xcalcf:feature name="microsoft.com:LET_WF"/>
-        <xcalcf:feature name="microsoft.com:LAMBDA_WF"/>
-        <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
+    </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
     </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="20" uniqueCount="16">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="21">
   <si>
     <t>CPF</t>
   </si>
@@ -53,18 +54,12 @@
     <t>Treinamento/Curso</t>
   </si>
   <si>
-    <t>Data de Conclusão</t>
-  </si>
-  <si>
     <t>Mariana Carolina dos Santos</t>
   </si>
   <si>
     <t>BPF</t>
   </si>
   <si>
-    <t>13/08/2026</t>
-  </si>
-  <si>
     <t>Jair Alberto Gonçalves</t>
   </si>
   <si>
@@ -83,14 +78,38 @@
     <t>Heloisa MKT</t>
   </si>
   <si>
-    <t>15/07/2025</t>
+    <t>Mês</t>
+  </si>
+  <si>
+    <t>Dia</t>
+  </si>
+  <si>
+    <t>Ano</t>
+  </si>
+  <si>
+    <t>Agosto</t>
+  </si>
+  <si>
+    <t>Carga</t>
+  </si>
+  <si>
+    <t>1h30</t>
+  </si>
+  <si>
+    <t>10h30</t>
+  </si>
+  <si>
+    <t>Eduardo Mondini</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <numFmts count="1">
+    <numFmt numFmtId="165" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+  </numFmts>
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -119,12 +138,15 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="4">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="14" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center" indent="1"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
@@ -407,19 +429,19 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:F7"/>
-  <sheetFormatPr defaultColWidth="18.42578125" defaultRowHeight="14.45"/>
+  <dimension ref="A1:I8"/>
+  <sheetFormatPr defaultColWidth="18.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.5703125" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.85546875" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="43.42578125" style="1" customWidth="1"/>
-    <col min="5" max="5" width="23.140625" style="1" customWidth="1"/>
-    <col min="6" max="6" width="18.7109375" style="1" bestFit="1" customWidth="1"/>
-    <col min="7" max="16384" width="18.42578125" style="1"/>
+    <col min="1" max="1" width="14.54296875" style="1" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="43.453125" style="1" customWidth="1"/>
+    <col min="5" max="5" width="23.1796875" style="1" customWidth="1"/>
+    <col min="6" max="6" width="18.7265625" style="1" bestFit="1" customWidth="1"/>
+    <col min="7" max="16384" width="18.453125" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:6">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -436,10 +458,19 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>5</v>
-      </c>
-    </row>
-    <row r="2" spans="1:6">
+        <v>14</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="H1" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="I1" s="1" t="s">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="1">
         <v>47167140805</v>
       </c>
@@ -447,20 +478,29 @@
         <v>2000</v>
       </c>
       <c r="C2" s="1" t="str">
-        <f>RIGHT(A2,4)&amp;B2</f>
+        <f t="shared" ref="C2:C8" si="0">RIGHT(A2,4)&amp;B2</f>
         <v>08052000</v>
       </c>
       <c r="D2" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="E2" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="E2" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F2" s="1" t="s">
-        <v>8</v>
-      </c>
-    </row>
-    <row r="3" spans="1:6">
+      <c r="F2" s="1">
+        <v>13</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H2" s="1">
+        <v>2026</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="1">
         <v>39096508807</v>
       </c>
@@ -468,20 +508,29 @@
         <v>1990</v>
       </c>
       <c r="C3" s="1" t="str">
-        <f>RIGHT(A3,4)&amp;B3</f>
+        <f t="shared" si="0"/>
         <v>88071990</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="F3" s="2">
-        <v>46248</v>
-      </c>
-    </row>
-    <row r="4" spans="1:6">
+        <v>14</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H3" s="1">
+        <v>2026</v>
+      </c>
+      <c r="I3" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="1">
         <v>48953912806</v>
       </c>
@@ -489,20 +538,29 @@
         <v>2000</v>
       </c>
       <c r="C4" s="1" t="str">
-        <f>RIGHT(A4,4)&amp;B4</f>
+        <f t="shared" si="0"/>
         <v>28062000</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="F4" s="2">
-        <v>46248</v>
-      </c>
-    </row>
-    <row r="5" spans="1:6">
+        <v>14</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H4" s="1">
+        <v>2026</v>
+      </c>
+      <c r="I4" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="1">
         <v>39096508807</v>
       </c>
@@ -510,20 +568,29 @@
         <v>1990</v>
       </c>
       <c r="C5" s="1" t="str">
-        <f>RIGHT(A5,4)&amp;B5</f>
+        <f t="shared" si="0"/>
         <v>88071990</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>9</v>
+        <v>7</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F5" s="2">
-        <v>46248</v>
-      </c>
-    </row>
-    <row r="6" spans="1:6">
+        <v>13</v>
+      </c>
+      <c r="G5" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H5" s="1">
+        <v>2026</v>
+      </c>
+      <c r="I5" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="1">
         <v>37257970807</v>
       </c>
@@ -531,20 +598,29 @@
         <v>2000</v>
       </c>
       <c r="C6" s="1" t="str">
-        <f>RIGHT(A6,4)&amp;B6</f>
+        <f t="shared" si="0"/>
         <v>08072000</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="E6" s="1" t="s">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F6" s="2">
-        <v>46248</v>
-      </c>
-    </row>
-    <row r="7" spans="1:6">
+        <v>12</v>
+      </c>
+      <c r="G6" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H6" s="1">
+        <v>2026</v>
+      </c>
+      <c r="I6" s="3" t="s">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="1">
         <v>53316429859</v>
       </c>
@@ -552,17 +628,56 @@
         <v>2003</v>
       </c>
       <c r="C7" s="1" t="str">
-        <f>RIGHT(A7,4)&amp;B7</f>
+        <f t="shared" si="0"/>
         <v>98592003</v>
       </c>
       <c r="D7" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="E7" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F7" s="2">
         <v>14</v>
       </c>
-      <c r="E7" s="1" t="s">
-        <v>7</v>
-      </c>
-      <c r="F7" s="2" t="s">
-        <v>15</v>
+      <c r="G7" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H7" s="1">
+        <v>2026</v>
+      </c>
+      <c r="I7" s="3" t="s">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A8" s="1">
+        <v>12345678900</v>
+      </c>
+      <c r="B8" s="1">
+        <v>2000</v>
+      </c>
+      <c r="C8" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>89002000</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="E8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="F8" s="1">
+        <v>14</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="H8" s="1">
+        <v>2026</v>
+      </c>
+      <c r="I8" s="1" t="s">
+        <v>18</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza texto do e-mail de certificado e planilha modelo
- server/index.js: novo texto do corpo do e-mail (saudação, sem
  menção fixa de carga horária no corpo)
- assets/Modelo Certificado.xlsx: atualiza dados
- .gitignore: ignora logs do servidor local

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/Modelo Certificado.xlsx
+++ b/assets/Modelo Certificado.xlsx
@@ -8,7 +8,8 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://atlheticanutrition-my.sharepoint.com/personal/digital_platforms_nutramerica_com_br/Documents/DEV/TOTEN CERTIFICADO/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="66" documentId="8_{42677D5F-0A19-4617-994D-499172CF4C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{39226497-9F1D-4A34-A42C-E5A2AB1BE553}"/>
+  <xr:revisionPtr revIDLastSave="82" documentId="8_{42677D5F-0A19-4617-994D-499172CF4C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{1249D7CD-BB04-4648-ABA2-20CD96A8864E}"/>
+  <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="NqJ3wjgx3cR7sVkcjUgjQiZb+1Evdvoja7xCh7UBIlMuCccWPD+KD7gWt7OFG5fGKNERamv/HrY1kCOk7uqHKQ==" workbookSaltValue="QbyEgElAzcOx3LPBthQYDA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="8150" yWindow="2570" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -37,7 +38,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="37" uniqueCount="21">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="41" uniqueCount="22">
   <si>
     <t>CPF</t>
   </si>
@@ -54,12 +55,30 @@
     <t>Treinamento/Curso</t>
   </si>
   <si>
+    <t>Dia</t>
+  </si>
+  <si>
+    <t>Mês</t>
+  </si>
+  <si>
+    <t>Ano</t>
+  </si>
+  <si>
+    <t>Carga</t>
+  </si>
+  <si>
     <t>Mariana Carolina dos Santos</t>
   </si>
   <si>
     <t>BPF</t>
   </si>
   <si>
+    <t>Agosto</t>
+  </si>
+  <si>
+    <t>1h30</t>
+  </si>
+  <si>
     <t>Jair Alberto Gonçalves</t>
   </si>
   <si>
@@ -78,28 +97,13 @@
     <t>Heloisa MKT</t>
   </si>
   <si>
-    <t>Mês</t>
-  </si>
-  <si>
-    <t>Dia</t>
-  </si>
-  <si>
-    <t>Ano</t>
-  </si>
-  <si>
-    <t>Agosto</t>
-  </si>
-  <si>
-    <t>Carga</t>
-  </si>
-  <si>
-    <t>1h30</t>
-  </si>
-  <si>
     <t>10h30</t>
   </si>
   <si>
     <t>Eduardo Mondini</t>
+  </si>
+  <si>
+    <t>t.i.</t>
   </si>
 </sst>
 </file>
@@ -107,7 +111,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
+    <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
   <fonts count="1" x14ac:knownFonts="1">
     <font>
@@ -138,15 +142,12 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center" indent="1"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="1"/>
     </xf>
   </cellXfs>
@@ -429,11 +430,11 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:I9"/>
   <sheetFormatPr defaultColWidth="18.453125" defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="14.54296875" style="1" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.81640625" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="14.54296875" style="1" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="19.81640625" style="1" hidden="1" customWidth="1"/>
     <col min="3" max="3" width="19.7265625" style="1" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="43.453125" style="1" customWidth="1"/>
     <col min="5" max="5" width="23.1796875" style="1" customWidth="1"/>
@@ -458,16 +459,16 @@
         <v>4</v>
       </c>
       <c r="F1" s="1" t="s">
-        <v>14</v>
+        <v>5</v>
       </c>
       <c r="G1" s="1" t="s">
-        <v>13</v>
+        <v>6</v>
       </c>
       <c r="H1" s="1" t="s">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="I1" s="1" t="s">
-        <v>17</v>
+        <v>8</v>
       </c>
     </row>
     <row r="2" spans="1:9" x14ac:dyDescent="0.35">
@@ -478,26 +479,26 @@
         <v>2000</v>
       </c>
       <c r="C2" s="1" t="str">
-        <f t="shared" ref="C2:C8" si="0">RIGHT(A2,4)&amp;B2</f>
+        <f t="shared" ref="C2:C9" si="0">RIGHT(A2,4)&amp;B2</f>
         <v>08052000</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>5</v>
+        <v>9</v>
       </c>
       <c r="E2" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F2" s="1">
         <v>13</v>
       </c>
       <c r="G2" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H2" s="1">
         <v>2026</v>
       </c>
-      <c r="I2" s="3" t="s">
-        <v>18</v>
+      <c r="I2" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="3" spans="1:9" x14ac:dyDescent="0.35">
@@ -512,22 +513,22 @@
         <v>88071990</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E3" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="F3" s="2">
         <v>14</v>
       </c>
+      <c r="F3" s="1">
+        <v>14</v>
+      </c>
       <c r="G3" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H3" s="1">
         <v>2026</v>
       </c>
-      <c r="I3" s="3" t="s">
-        <v>18</v>
+      <c r="I3" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="4" spans="1:9" x14ac:dyDescent="0.35">
@@ -542,22 +543,22 @@
         <v>28062000</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>9</v>
+        <v>15</v>
       </c>
       <c r="E4" s="1" t="s">
-        <v>10</v>
-      </c>
-      <c r="F4" s="2">
+        <v>16</v>
+      </c>
+      <c r="F4" s="1">
         <v>14</v>
       </c>
       <c r="G4" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H4" s="1">
         <v>2026</v>
       </c>
-      <c r="I4" s="3" t="s">
-        <v>18</v>
+      <c r="I4" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="5" spans="1:9" x14ac:dyDescent="0.35">
@@ -572,22 +573,22 @@
         <v>88071990</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>7</v>
+        <v>13</v>
       </c>
       <c r="E5" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F5" s="2">
+        <v>10</v>
+      </c>
+      <c r="F5" s="1">
         <v>13</v>
       </c>
       <c r="G5" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H5" s="1">
         <v>2026</v>
       </c>
-      <c r="I5" s="3" t="s">
-        <v>18</v>
+      <c r="I5" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="6" spans="1:9" x14ac:dyDescent="0.35">
@@ -602,22 +603,22 @@
         <v>08072000</v>
       </c>
       <c r="D6" s="1" t="s">
+        <v>17</v>
+      </c>
+      <c r="E6" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="F6" s="1">
+        <v>12</v>
+      </c>
+      <c r="G6" s="1" t="s">
         <v>11</v>
-      </c>
-      <c r="E6" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F6" s="2">
-        <v>12</v>
-      </c>
-      <c r="G6" s="1" t="s">
-        <v>16</v>
       </c>
       <c r="H6" s="1">
         <v>2026</v>
       </c>
-      <c r="I6" s="3" t="s">
-        <v>18</v>
+      <c r="I6" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
     <row r="7" spans="1:9" x14ac:dyDescent="0.35">
@@ -632,21 +633,21 @@
         <v>98592003</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="E7" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="F7" s="2">
+        <v>10</v>
+      </c>
+      <c r="F7" s="1">
         <v>14</v>
       </c>
       <c r="G7" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H7" s="1">
         <v>2026</v>
       </c>
-      <c r="I7" s="3" t="s">
+      <c r="I7" s="2" t="s">
         <v>19</v>
       </c>
     </row>
@@ -665,22 +666,56 @@
         <v>20</v>
       </c>
       <c r="E8" s="1" t="s">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F8" s="1">
         <v>14</v>
       </c>
       <c r="G8" s="1" t="s">
-        <v>16</v>
+        <v>11</v>
       </c>
       <c r="H8" s="1">
         <v>2026</v>
       </c>
       <c r="I8" s="1" t="s">
-        <v>18</v>
+        <v>12</v>
+      </c>
+    </row>
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A9" s="1">
+        <v>78945612300</v>
+      </c>
+      <c r="B9" s="1">
+        <v>2000</v>
+      </c>
+      <c r="C9" s="1" t="str">
+        <f t="shared" si="0"/>
+        <v>23002000</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="E9" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="F9" s="1">
+        <v>26</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>11</v>
+      </c>
+      <c r="H9" s="1">
+        <v>2026</v>
+      </c>
+      <c r="I9" s="2" t="s">
+        <v>12</v>
       </c>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="5mLEFixRyCIpcNbdS+3hmojikOW/T5RIV2+iyX+n9ZHRYkWKd1cRPAjHYqydZy5tSX/IAzOt2a+xlLm4EC8QgA==" saltValue="sPUFcXkno+CaQHFQDhxNeA==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1" selectUnlockedCells="1"/>
+  <protectedRanges>
+    <protectedRange sqref="C1:I1048576" name="Range1"/>
+  </protectedRanges>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Regenera certificados-data.js a partir da planilha atualizada (130 certificados)
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/Modelo Certificado.xlsx
+++ b/assets/Modelo Certificado.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30404"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://atlheticanutrition-my.sharepoint.com/personal/digital_platforms_nutramerica_com_br/Documents/DEV/TOTEN CERTIFICADO/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="308" documentId="8_{42677D5F-0A19-4617-994D-499172CF4C88}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{B964539E-2EA7-4F20-870C-268C7D761571}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="14_{855DC049-69AE-459E-A0C6-62EC7BE3C0C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="NqJ3wjgx3cR7sVkcjUgjQiZb+1Evdvoja7xCh7UBIlMuCccWPD+KD7gWt7OFG5fGKNERamv/HrY1kCOk7uqHKQ==" workbookSaltValue="QbyEgElAzcOx3LPBthQYDA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="8150" yWindow="2570" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -35,6 +35,9 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
@@ -493,7 +496,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="4">
+  <fonts count="4" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -941,22 +944,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I132"/>
-  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75"/>
+  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
   <cols>
-    <col min="1" max="1" width="16.140625" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.85546875" style="3" customWidth="1"/>
-    <col min="3" max="3" width="19.7109375" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.1796875" style="6" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="19.81640625" style="3" customWidth="1"/>
+    <col min="3" max="3" width="19.7265625" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.453125" style="3" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="67" style="3" customWidth="1"/>
-    <col min="6" max="9" width="9.5703125" style="3" customWidth="1"/>
-    <col min="10" max="14" width="9.140625" style="3"/>
-    <col min="15" max="15" width="34.140625" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="34.140625" style="3" customWidth="1"/>
+    <col min="6" max="9" width="9.54296875" style="3" customWidth="1"/>
+    <col min="10" max="14" width="9.1796875" style="3"/>
+    <col min="15" max="15" width="34.1796875" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="34.1796875" style="3" customWidth="1"/>
     <col min="17" max="17" width="37" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.140625" style="3"/>
+    <col min="18" max="16384" width="9.1796875" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9">
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -985,7 +988,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9">
+    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A2" s="8">
         <v>4349484469</v>
       </c>
@@ -993,7 +996,7 @@
         <v>1981</v>
       </c>
       <c r="C2" s="2" t="str">
-        <f>RIGHT(A2,4)&amp;B2</f>
+        <f t="shared" ref="C2:C33" si="0">RIGHT(A2,4)&amp;B2</f>
         <v>44691981</v>
       </c>
       <c r="D2" s="9" t="s">
@@ -1015,7 +1018,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:9">
+    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A3" s="8">
         <v>27672701878</v>
       </c>
@@ -1023,7 +1026,7 @@
         <v>1979</v>
       </c>
       <c r="C3" s="2" t="str">
-        <f>RIGHT(A3,4)&amp;B3</f>
+        <f t="shared" si="0"/>
         <v>18781979</v>
       </c>
       <c r="D3" s="9" t="s">
@@ -1045,7 +1048,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:9">
+    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A4" s="8">
         <v>35353327888</v>
       </c>
@@ -1053,7 +1056,7 @@
         <v>1987</v>
       </c>
       <c r="C4" s="2" t="str">
-        <f>RIGHT(A4,4)&amp;B4</f>
+        <f t="shared" si="0"/>
         <v>78881987</v>
       </c>
       <c r="D4" s="9" t="s">
@@ -1075,7 +1078,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:9">
+    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A5" s="8">
         <v>41197627855</v>
       </c>
@@ -1083,7 +1086,7 @@
         <v>1992</v>
       </c>
       <c r="C5" s="2" t="str">
-        <f>RIGHT(A5,4)&amp;B5</f>
+        <f t="shared" si="0"/>
         <v>78551992</v>
       </c>
       <c r="D5" s="9" t="s">
@@ -1105,7 +1108,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:9">
+    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A6" s="8">
         <v>53994007828</v>
       </c>
@@ -1113,7 +1116,7 @@
         <v>2005</v>
       </c>
       <c r="C6" s="2" t="str">
-        <f>RIGHT(A6,4)&amp;B6</f>
+        <f t="shared" si="0"/>
         <v>78282005</v>
       </c>
       <c r="D6" s="9" t="s">
@@ -1135,7 +1138,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:9">
+    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A7" s="8">
         <v>43876868807</v>
       </c>
@@ -1143,7 +1146,7 @@
         <v>1996</v>
       </c>
       <c r="C7" s="2" t="str">
-        <f>RIGHT(A7,4)&amp;B7</f>
+        <f t="shared" si="0"/>
         <v>88071996</v>
       </c>
       <c r="D7" s="9" t="s">
@@ -1165,7 +1168,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:9">
+    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A8" s="10">
         <v>42186704803</v>
       </c>
@@ -1173,7 +1176,7 @@
         <v>1996</v>
       </c>
       <c r="C8" s="2" t="str">
-        <f>RIGHT(A8,4)&amp;B8</f>
+        <f t="shared" si="0"/>
         <v>48031996</v>
       </c>
       <c r="D8" s="2" t="s">
@@ -1195,7 +1198,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:9">
+    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A9" s="1" t="s">
         <v>19</v>
       </c>
@@ -1203,7 +1206,7 @@
         <v>1997</v>
       </c>
       <c r="C9" s="2" t="str">
-        <f>RIGHT(A9,4)&amp;B9</f>
+        <f t="shared" si="0"/>
         <v>58801997</v>
       </c>
       <c r="D9" s="2" t="s">
@@ -1225,7 +1228,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:9">
+    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A10" s="8">
         <v>44666032860</v>
       </c>
@@ -1233,7 +1236,7 @@
         <v>1994</v>
       </c>
       <c r="C10" s="2" t="str">
-        <f>RIGHT(A10,4)&amp;B10</f>
+        <f t="shared" si="0"/>
         <v>28601994</v>
       </c>
       <c r="D10" s="9" t="s">
@@ -1255,7 +1258,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:9">
+    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A11" s="8">
         <v>46967903802</v>
       </c>
@@ -1263,7 +1266,7 @@
         <v>2007</v>
       </c>
       <c r="C11" s="2" t="str">
-        <f>RIGHT(A11,4)&amp;B11</f>
+        <f t="shared" si="0"/>
         <v>38022007</v>
       </c>
       <c r="D11" s="9" t="s">
@@ -1285,7 +1288,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
+    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A12" s="8">
         <v>47193017896</v>
       </c>
@@ -1293,7 +1296,7 @@
         <v>2000</v>
       </c>
       <c r="C12" s="2" t="str">
-        <f>RIGHT(A12,4)&amp;B12</f>
+        <f t="shared" si="0"/>
         <v>78962000</v>
       </c>
       <c r="D12" s="9" t="s">
@@ -1315,7 +1318,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:9">
+    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A13" s="8">
         <v>34687383823</v>
       </c>
@@ -1323,7 +1326,7 @@
         <v>2001</v>
       </c>
       <c r="C13" s="2" t="str">
-        <f>RIGHT(A13,4)&amp;B13</f>
+        <f t="shared" si="0"/>
         <v>38232001</v>
       </c>
       <c r="D13" s="9" t="s">
@@ -1345,7 +1348,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:9">
+    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A14" s="8">
         <v>37835487802</v>
       </c>
@@ -1353,7 +1356,7 @@
         <v>1987</v>
       </c>
       <c r="C14" s="2" t="str">
-        <f>RIGHT(A14,4)&amp;B14</f>
+        <f t="shared" si="0"/>
         <v>78021987</v>
       </c>
       <c r="D14" s="9" t="s">
@@ -1375,7 +1378,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:9">
+    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A15" s="7" t="s">
         <v>26</v>
       </c>
@@ -1383,7 +1386,7 @@
         <v>1982</v>
       </c>
       <c r="C15" s="2" t="str">
-        <f>RIGHT(A15,4)&amp;B15</f>
+        <f t="shared" si="0"/>
         <v>97841982</v>
       </c>
       <c r="D15" s="5" t="s">
@@ -1405,7 +1408,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:9">
+    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A16" s="8">
         <v>48954491812</v>
       </c>
@@ -1413,7 +1416,7 @@
         <v>1997</v>
       </c>
       <c r="C16" s="2" t="str">
-        <f>RIGHT(A16,4)&amp;B16</f>
+        <f t="shared" si="0"/>
         <v>18121997</v>
       </c>
       <c r="D16" s="9" t="s">
@@ -1435,7 +1438,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:9">
+    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A17" s="8">
         <v>46997604811</v>
       </c>
@@ -1443,7 +1446,7 @@
         <v>1995</v>
       </c>
       <c r="C17" s="2" t="str">
-        <f>RIGHT(A17,4)&amp;B17</f>
+        <f t="shared" si="0"/>
         <v>48111995</v>
       </c>
       <c r="D17" s="9" t="s">
@@ -1465,7 +1468,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:9">
+    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A18" s="8">
         <v>36945656802</v>
       </c>
@@ -1473,7 +1476,7 @@
         <v>1988</v>
       </c>
       <c r="C18" s="2" t="str">
-        <f>RIGHT(A18,4)&amp;B18</f>
+        <f t="shared" si="0"/>
         <v>68021988</v>
       </c>
       <c r="D18" s="9" t="s">
@@ -1495,7 +1498,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:9">
+    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A19" s="10">
         <v>26920249820</v>
       </c>
@@ -1503,7 +1506,7 @@
         <v>1979</v>
       </c>
       <c r="C19" s="2" t="str">
-        <f>RIGHT(A19,4)&amp;B19</f>
+        <f t="shared" si="0"/>
         <v>98201979</v>
       </c>
       <c r="D19" s="5" t="s">
@@ -1525,7 +1528,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:9">
+    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A20" s="8">
         <v>25495474899</v>
       </c>
@@ -1533,7 +1536,7 @@
         <v>1971</v>
       </c>
       <c r="C20" s="2" t="str">
-        <f>RIGHT(A20,4)&amp;B20</f>
+        <f t="shared" si="0"/>
         <v>48991971</v>
       </c>
       <c r="D20" s="9" t="s">
@@ -1555,11 +1558,11 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:9">
+    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A21" s="1"/>
       <c r="B21" s="2"/>
       <c r="C21" s="2" t="str">
-        <f>RIGHT(A21,4)&amp;B21</f>
+        <f t="shared" si="0"/>
         <v/>
       </c>
       <c r="D21" s="2" t="s">
@@ -1581,7 +1584,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:9">
+    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A22" s="8">
         <v>31230944800</v>
       </c>
@@ -1589,7 +1592,7 @@
         <v>1977</v>
       </c>
       <c r="C22" s="2" t="str">
-        <f>RIGHT(A22,4)&amp;B22</f>
+        <f t="shared" si="0"/>
         <v>48001977</v>
       </c>
       <c r="D22" s="9" t="s">
@@ -1611,7 +1614,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:9">
+    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A23" s="8">
         <v>50155292870</v>
       </c>
@@ -1619,7 +1622,7 @@
         <v>2000</v>
       </c>
       <c r="C23" s="2" t="str">
-        <f>RIGHT(A23,4)&amp;B23</f>
+        <f t="shared" si="0"/>
         <v>28702000</v>
       </c>
       <c r="D23" s="9" t="s">
@@ -1641,7 +1644,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:9">
+    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A24" s="8">
         <v>46476927876</v>
       </c>
@@ -1649,7 +1652,7 @@
         <v>1996</v>
       </c>
       <c r="C24" s="2" t="str">
-        <f>RIGHT(A24,4)&amp;B24</f>
+        <f t="shared" si="0"/>
         <v>78761996</v>
       </c>
       <c r="D24" s="9" t="s">
@@ -1671,7 +1674,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="1:9">
+    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A25" s="8">
         <v>42039343890</v>
       </c>
@@ -1679,7 +1682,7 @@
         <v>1993</v>
       </c>
       <c r="C25" s="2" t="str">
-        <f>RIGHT(A25,4)&amp;B25</f>
+        <f t="shared" si="0"/>
         <v>38901993</v>
       </c>
       <c r="D25" s="9" t="s">
@@ -1701,7 +1704,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="1:9">
+    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A26" s="8">
         <v>44891522801</v>
       </c>
@@ -1709,7 +1712,7 @@
         <v>1996</v>
       </c>
       <c r="C26" s="2" t="str">
-        <f>RIGHT(A26,4)&amp;B26</f>
+        <f t="shared" si="0"/>
         <v>28011996</v>
       </c>
       <c r="D26" s="9" t="s">
@@ -1731,7 +1734,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:9">
+    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A27" s="8">
         <v>36377720866</v>
       </c>
@@ -1739,7 +1742,7 @@
         <v>1992</v>
       </c>
       <c r="C27" s="2" t="str">
-        <f>RIGHT(A27,4)&amp;B27</f>
+        <f t="shared" si="0"/>
         <v>08661992</v>
       </c>
       <c r="D27" s="9" t="s">
@@ -1761,7 +1764,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:9">
+    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A28" s="8">
         <v>52750031885</v>
       </c>
@@ -1769,7 +1772,7 @@
         <v>2003</v>
       </c>
       <c r="C28" s="2" t="str">
-        <f>RIGHT(A28,4)&amp;B28</f>
+        <f t="shared" si="0"/>
         <v>18852003</v>
       </c>
       <c r="D28" s="9" t="s">
@@ -1791,7 +1794,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="29" spans="1:9">
+    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A29" s="11">
         <v>39974249856</v>
       </c>
@@ -1799,7 +1802,7 @@
         <v>1991</v>
       </c>
       <c r="C29" s="2" t="str">
-        <f>RIGHT(A29,4)&amp;B29</f>
+        <f t="shared" si="0"/>
         <v>98561991</v>
       </c>
       <c r="D29" s="2" t="s">
@@ -1821,7 +1824,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:9">
+    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A30" s="8">
         <v>37714454857</v>
       </c>
@@ -1829,7 +1832,7 @@
         <v>1995</v>
       </c>
       <c r="C30" s="2" t="str">
-        <f>RIGHT(A30,4)&amp;B30</f>
+        <f t="shared" si="0"/>
         <v>48571995</v>
       </c>
       <c r="D30" s="9" t="s">
@@ -1851,7 +1854,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:9">
+    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A31" s="8">
         <v>37606164886</v>
       </c>
@@ -1859,7 +1862,7 @@
         <v>1995</v>
       </c>
       <c r="C31" s="2" t="str">
-        <f>RIGHT(A31,4)&amp;B31</f>
+        <f t="shared" si="0"/>
         <v>48861995</v>
       </c>
       <c r="D31" s="9" t="s">
@@ -1881,7 +1884,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:9">
+    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A32" s="8">
         <v>33864275881</v>
       </c>
@@ -1889,7 +1892,7 @@
         <v>1982</v>
       </c>
       <c r="C32" s="2" t="str">
-        <f>RIGHT(A32,4)&amp;B32</f>
+        <f t="shared" si="0"/>
         <v>58811982</v>
       </c>
       <c r="D32" s="9" t="s">
@@ -1911,7 +1914,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="33" spans="1:9">
+    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A33" s="8">
         <v>35971031899</v>
       </c>
@@ -1919,7 +1922,7 @@
         <v>1988</v>
       </c>
       <c r="C33" s="2" t="str">
-        <f>RIGHT(A33,4)&amp;B33</f>
+        <f t="shared" si="0"/>
         <v>18991988</v>
       </c>
       <c r="D33" s="9" t="s">
@@ -1941,7 +1944,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:9">
+    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A34" s="8">
         <v>37383312805</v>
       </c>
@@ -1949,7 +1952,7 @@
         <v>1987</v>
       </c>
       <c r="C34" s="2" t="str">
-        <f>RIGHT(A34,4)&amp;B34</f>
+        <f t="shared" ref="C34:C65" si="1">RIGHT(A34,4)&amp;B34</f>
         <v>28051987</v>
       </c>
       <c r="D34" s="9" t="s">
@@ -1971,7 +1974,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:9">
+    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A35" s="8">
         <v>35989473800</v>
       </c>
@@ -1979,7 +1982,7 @@
         <v>2002</v>
       </c>
       <c r="C35" s="2" t="str">
-        <f>RIGHT(A35,4)&amp;B35</f>
+        <f t="shared" si="1"/>
         <v>38002002</v>
       </c>
       <c r="D35" s="9" t="s">
@@ -2001,7 +2004,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="36" spans="1:9">
+    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A36" s="8">
         <v>47128318801</v>
       </c>
@@ -2009,7 +2012,7 @@
         <v>1987</v>
       </c>
       <c r="C36" s="2" t="str">
-        <f>RIGHT(A36,4)&amp;B36</f>
+        <f t="shared" si="1"/>
         <v>88011987</v>
       </c>
       <c r="D36" s="9" t="s">
@@ -2031,7 +2034,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="37" spans="1:9">
+    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A37" s="8">
         <v>53700882840</v>
       </c>
@@ -2039,7 +2042,7 @@
         <v>2007</v>
       </c>
       <c r="C37" s="2" t="str">
-        <f>RIGHT(A37,4)&amp;B37</f>
+        <f t="shared" si="1"/>
         <v>28402007</v>
       </c>
       <c r="D37" s="9" t="s">
@@ -2061,7 +2064,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="38" spans="1:9">
+    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A38" s="8">
         <v>43736502842</v>
       </c>
@@ -2069,7 +2072,7 @@
         <v>1992</v>
       </c>
       <c r="C38" s="2" t="str">
-        <f>RIGHT(A38,4)&amp;B38</f>
+        <f t="shared" si="1"/>
         <v>28421992</v>
       </c>
       <c r="D38" s="9" t="s">
@@ -2091,7 +2094,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:9">
+    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A39" s="8">
         <v>45884235844</v>
       </c>
@@ -2099,7 +2102,7 @@
         <v>1996</v>
       </c>
       <c r="C39" s="2" t="str">
-        <f>RIGHT(A39,4)&amp;B39</f>
+        <f t="shared" si="1"/>
         <v>58441996</v>
       </c>
       <c r="D39" s="9" t="s">
@@ -2121,7 +2124,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="40" spans="1:9">
+    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A40" s="8">
         <v>44020167893</v>
       </c>
@@ -2129,7 +2132,7 @@
         <v>1996</v>
       </c>
       <c r="C40" s="2" t="str">
-        <f>RIGHT(A40,4)&amp;B40</f>
+        <f t="shared" si="1"/>
         <v>78931996</v>
       </c>
       <c r="D40" s="9" t="s">
@@ -2151,7 +2154,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="41" spans="1:9">
+    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A41" s="8">
         <v>33434644814</v>
       </c>
@@ -2159,7 +2162,7 @@
         <v>1985</v>
       </c>
       <c r="C41" s="2" t="str">
-        <f>RIGHT(A41,4)&amp;B41</f>
+        <f t="shared" si="1"/>
         <v>48141985</v>
       </c>
       <c r="D41" s="9" t="s">
@@ -2181,7 +2184,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="42" spans="1:9">
+    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A42" s="8">
         <v>43139451806</v>
       </c>
@@ -2189,7 +2192,7 @@
         <v>1995</v>
       </c>
       <c r="C42" s="2" t="str">
-        <f>RIGHT(A42,4)&amp;B42</f>
+        <f t="shared" si="1"/>
         <v>18061995</v>
       </c>
       <c r="D42" s="9" t="s">
@@ -2211,7 +2214,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="43" spans="1:9">
+    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A43" s="10">
         <v>24944634838</v>
       </c>
@@ -2219,7 +2222,7 @@
         <v>1976</v>
       </c>
       <c r="C43" s="2" t="str">
-        <f>RIGHT(A43,4)&amp;B43</f>
+        <f t="shared" si="1"/>
         <v>48381976</v>
       </c>
       <c r="D43" s="2" t="s">
@@ -2241,7 +2244,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="44" spans="1:9">
+    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A44" s="8">
         <v>28801880839</v>
       </c>
@@ -2249,7 +2252,7 @@
         <v>1981</v>
       </c>
       <c r="C44" s="2" t="str">
-        <f>RIGHT(A44,4)&amp;B44</f>
+        <f t="shared" si="1"/>
         <v>08391981</v>
       </c>
       <c r="D44" s="9" t="s">
@@ -2271,7 +2274,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="45" spans="1:9">
+    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A45" s="8">
         <v>41667619861</v>
       </c>
@@ -2279,7 +2282,7 @@
         <v>2003</v>
       </c>
       <c r="C45" s="2" t="str">
-        <f>RIGHT(A45,4)&amp;B45</f>
+        <f t="shared" si="1"/>
         <v>98612003</v>
       </c>
       <c r="D45" s="9" t="s">
@@ -2301,7 +2304,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="46" spans="1:9">
+    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A46" s="8">
         <v>10838890440</v>
       </c>
@@ -2309,7 +2312,7 @@
         <v>1993</v>
       </c>
       <c r="C46" s="2" t="str">
-        <f>RIGHT(A46,4)&amp;B46</f>
+        <f t="shared" si="1"/>
         <v>04401993</v>
       </c>
       <c r="D46" s="9" t="s">
@@ -2331,7 +2334,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="47" spans="1:9">
+    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A47" s="8">
         <v>43118475803</v>
       </c>
@@ -2339,7 +2342,7 @@
         <v>1996</v>
       </c>
       <c r="C47" s="2" t="str">
-        <f>RIGHT(A47,4)&amp;B47</f>
+        <f t="shared" si="1"/>
         <v>58031996</v>
       </c>
       <c r="D47" s="9" t="s">
@@ -2361,7 +2364,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="48" spans="1:9">
+    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A48" s="8">
         <v>47440294858</v>
       </c>
@@ -2369,7 +2372,7 @@
         <v>1998</v>
       </c>
       <c r="C48" s="2" t="str">
-        <f>RIGHT(A48,4)&amp;B48</f>
+        <f t="shared" si="1"/>
         <v>48581998</v>
       </c>
       <c r="D48" s="9" t="s">
@@ -2391,7 +2394,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="49" spans="1:9">
+    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A49" s="1" t="s">
         <v>61</v>
       </c>
@@ -2399,7 +2402,7 @@
         <v>1978</v>
       </c>
       <c r="C49" s="2" t="str">
-        <f>RIGHT(A49,4)&amp;B49</f>
+        <f t="shared" si="1"/>
         <v>08671978</v>
       </c>
       <c r="D49" s="2" t="s">
@@ -2421,7 +2424,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="50" spans="1:9">
+    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A50" s="8">
         <v>37257970807</v>
       </c>
@@ -2429,7 +2432,7 @@
         <v>2000</v>
       </c>
       <c r="C50" s="2" t="str">
-        <f>RIGHT(A50,4)&amp;B50</f>
+        <f t="shared" si="1"/>
         <v>08072000</v>
       </c>
       <c r="D50" s="9" t="s">
@@ -2451,7 +2454,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="51" spans="1:9">
+    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A51" s="8">
         <v>42247533833</v>
       </c>
@@ -2459,7 +2462,7 @@
         <v>1992</v>
       </c>
       <c r="C51" s="2" t="str">
-        <f>RIGHT(A51,4)&amp;B51</f>
+        <f t="shared" si="1"/>
         <v>38331992</v>
       </c>
       <c r="D51" s="9" t="s">
@@ -2481,7 +2484,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="52" spans="1:9">
+    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A52" s="8">
         <v>45367371892</v>
       </c>
@@ -2489,7 +2492,7 @@
         <v>1995</v>
       </c>
       <c r="C52" s="2" t="str">
-        <f>RIGHT(A52,4)&amp;B52</f>
+        <f t="shared" si="1"/>
         <v>18921995</v>
       </c>
       <c r="D52" s="9" t="s">
@@ -2511,7 +2514,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="53" spans="1:9">
+    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A53" s="8">
         <v>44896404807</v>
       </c>
@@ -2519,7 +2522,7 @@
         <v>2002</v>
       </c>
       <c r="C53" s="2" t="str">
-        <f>RIGHT(A53,4)&amp;B53</f>
+        <f t="shared" si="1"/>
         <v>48072002</v>
       </c>
       <c r="D53" s="9" t="s">
@@ -2541,7 +2544,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="54" spans="1:9">
+    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A54" s="8">
         <v>42659165890</v>
       </c>
@@ -2549,7 +2552,7 @@
         <v>1994</v>
       </c>
       <c r="C54" s="2" t="str">
-        <f>RIGHT(A54,4)&amp;B54</f>
+        <f t="shared" si="1"/>
         <v>58901994</v>
       </c>
       <c r="D54" s="9" t="s">
@@ -2571,7 +2574,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="55" spans="1:9">
+    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A55" s="8">
         <v>36526421806</v>
       </c>
@@ -2579,7 +2582,7 @@
         <v>1987</v>
       </c>
       <c r="C55" s="2" t="str">
-        <f>RIGHT(A55,4)&amp;B55</f>
+        <f t="shared" si="1"/>
         <v>18061987</v>
       </c>
       <c r="D55" s="9" t="s">
@@ -2601,7 +2604,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="56" spans="1:9">
+    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A56" s="8">
         <v>53703468874</v>
       </c>
@@ -2609,7 +2612,7 @@
         <v>2006</v>
       </c>
       <c r="C56" s="2" t="str">
-        <f>RIGHT(A56,4)&amp;B56</f>
+        <f t="shared" si="1"/>
         <v>88742006</v>
       </c>
       <c r="D56" s="9" t="s">
@@ -2631,7 +2634,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="57" spans="1:9">
+    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A57" s="8">
         <v>49193907850</v>
       </c>
@@ -2639,7 +2642,7 @@
         <v>2003</v>
       </c>
       <c r="C57" s="2" t="str">
-        <f>RIGHT(A57,4)&amp;B57</f>
+        <f t="shared" si="1"/>
         <v>78502003</v>
       </c>
       <c r="D57" s="9" t="s">
@@ -2661,7 +2664,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="58" spans="1:9">
+    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A58" s="8">
         <v>51369270895</v>
       </c>
@@ -2669,7 +2672,7 @@
         <v>2003</v>
       </c>
       <c r="C58" s="2" t="str">
-        <f>RIGHT(A58,4)&amp;B58</f>
+        <f t="shared" si="1"/>
         <v>08952003</v>
       </c>
       <c r="D58" s="9" t="s">
@@ -2691,7 +2694,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="59" spans="1:9">
+    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A59" s="8">
         <v>53316429859</v>
       </c>
@@ -2699,7 +2702,7 @@
         <v>2003</v>
       </c>
       <c r="C59" s="2" t="str">
-        <f>RIGHT(A59,4)&amp;B59</f>
+        <f t="shared" si="1"/>
         <v>98592003</v>
       </c>
       <c r="D59" s="9" t="s">
@@ -2721,7 +2724,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="60" spans="1:9">
+    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A60" s="8">
         <v>27953697882</v>
       </c>
@@ -2729,7 +2732,7 @@
         <v>1977</v>
       </c>
       <c r="C60" s="2" t="str">
-        <f>RIGHT(A60,4)&amp;B60</f>
+        <f t="shared" si="1"/>
         <v>78821977</v>
       </c>
       <c r="D60" s="9" t="s">
@@ -2751,7 +2754,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="61" spans="1:9">
+    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A61" s="8">
         <v>50511623801</v>
       </c>
@@ -2759,7 +2762,7 @@
         <v>2008</v>
       </c>
       <c r="C61" s="2" t="str">
-        <f>RIGHT(A61,4)&amp;B61</f>
+        <f t="shared" si="1"/>
         <v>38012008</v>
       </c>
       <c r="D61" s="17" t="s">
@@ -2781,7 +2784,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="62" spans="1:9">
+    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A62" s="8">
         <v>39984951855</v>
       </c>
@@ -2789,7 +2792,7 @@
         <v>1991</v>
       </c>
       <c r="C62" s="2" t="str">
-        <f>RIGHT(A62,4)&amp;B62</f>
+        <f t="shared" si="1"/>
         <v>18551991</v>
       </c>
       <c r="D62" s="9" t="s">
@@ -2811,7 +2814,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="63" spans="1:9">
+    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A63" s="1" t="s">
         <v>76</v>
       </c>
@@ -2819,7 +2822,7 @@
         <v>1990</v>
       </c>
       <c r="C63" s="2" t="str">
-        <f>RIGHT(A63,4)&amp;B63</f>
+        <f t="shared" si="1"/>
         <v>88071990</v>
       </c>
       <c r="D63" s="14" t="s">
@@ -2841,7 +2844,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="64" spans="1:9">
+    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A64" s="8">
         <v>35440649875</v>
       </c>
@@ -2849,7 +2852,7 @@
         <v>1990</v>
       </c>
       <c r="C64" s="2" t="str">
-        <f>RIGHT(A64,4)&amp;B64</f>
+        <f t="shared" si="1"/>
         <v>98751990</v>
       </c>
       <c r="D64" s="9" t="s">
@@ -2871,7 +2874,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="65" spans="1:9">
+    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A65" s="14">
         <v>16716444840</v>
       </c>
@@ -2879,7 +2882,7 @@
         <v>1974</v>
       </c>
       <c r="C65" s="2" t="str">
-        <f>RIGHT(A65,4)&amp;B65</f>
+        <f t="shared" si="1"/>
         <v>48401974</v>
       </c>
       <c r="D65" s="14" t="s">
@@ -2901,7 +2904,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="66" spans="1:9">
+    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A66" s="8">
         <v>38214626803</v>
       </c>
@@ -2909,7 +2912,7 @@
         <v>1988</v>
       </c>
       <c r="C66" s="2" t="str">
-        <f>RIGHT(A66,4)&amp;B66</f>
+        <f t="shared" ref="C66:C97" si="2">RIGHT(A66,4)&amp;B66</f>
         <v>68031988</v>
       </c>
       <c r="D66" s="9" t="s">
@@ -2931,7 +2934,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="67" spans="1:9">
+    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A67" s="8">
         <v>57181251805</v>
       </c>
@@ -2939,7 +2942,7 @@
         <v>2004</v>
       </c>
       <c r="C67" s="2" t="str">
-        <f>RIGHT(A67,4)&amp;B67</f>
+        <f t="shared" si="2"/>
         <v>18052004</v>
       </c>
       <c r="D67" s="9" t="s">
@@ -2961,7 +2964,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="68" spans="1:9">
+    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A68" s="8">
         <v>41634273842</v>
       </c>
@@ -2969,7 +2972,7 @@
         <v>1992</v>
       </c>
       <c r="C68" s="2" t="str">
-        <f>RIGHT(A68,4)&amp;B68</f>
+        <f t="shared" si="2"/>
         <v>38421992</v>
       </c>
       <c r="D68" s="9" t="s">
@@ -2991,7 +2994,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="69" spans="1:9">
+    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A69" s="10">
         <v>22351070879</v>
       </c>
@@ -2999,7 +3002,7 @@
         <v>1981</v>
       </c>
       <c r="C69" s="2" t="str">
-        <f>RIGHT(A69,4)&amp;B69</f>
+        <f t="shared" si="2"/>
         <v>08791981</v>
       </c>
       <c r="D69" s="2" t="s">
@@ -3021,7 +3024,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="70" spans="1:9">
+    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A70" s="8">
         <v>25500655817</v>
       </c>
@@ -3029,7 +3032,7 @@
         <v>1977</v>
       </c>
       <c r="C70" s="2" t="str">
-        <f>RIGHT(A70,4)&amp;B70</f>
+        <f t="shared" si="2"/>
         <v>58171977</v>
       </c>
       <c r="D70" s="9" t="s">
@@ -3051,7 +3054,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="71" spans="1:9">
+    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A71" s="8">
         <v>39869048838</v>
       </c>
@@ -3059,7 +3062,7 @@
         <v>1992</v>
       </c>
       <c r="C71" s="2" t="str">
-        <f>RIGHT(A71,4)&amp;B71</f>
+        <f t="shared" si="2"/>
         <v>88381992</v>
       </c>
       <c r="D71" s="9" t="s">
@@ -3081,7 +3084,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="72" spans="1:9">
+    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A72" s="8">
         <v>52817337883</v>
       </c>
@@ -3089,7 +3092,7 @@
         <v>2002</v>
       </c>
       <c r="C72" s="2" t="str">
-        <f>RIGHT(A72,4)&amp;B72</f>
+        <f t="shared" si="2"/>
         <v>78832002</v>
       </c>
       <c r="D72" s="9" t="s">
@@ -3111,7 +3114,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="73" spans="1:9">
+    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A73" s="8">
         <v>16705635886</v>
       </c>
@@ -3119,7 +3122,7 @@
         <v>1976</v>
       </c>
       <c r="C73" s="2" t="str">
-        <f>RIGHT(A73,4)&amp;B73</f>
+        <f t="shared" si="2"/>
         <v>58861976</v>
       </c>
       <c r="D73" s="9" t="s">
@@ -3141,7 +3144,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="74" spans="1:9">
+    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A74" s="8">
         <v>52614291889</v>
       </c>
@@ -3149,7 +3152,7 @@
         <v>2005</v>
       </c>
       <c r="C74" s="2" t="str">
-        <f>RIGHT(A74,4)&amp;B74</f>
+        <f t="shared" si="2"/>
         <v>18892005</v>
       </c>
       <c r="D74" s="9" t="s">
@@ -3171,7 +3174,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="75" spans="1:9">
+    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A75" s="8">
         <v>37241029844</v>
       </c>
@@ -3179,7 +3182,7 @@
         <v>2005</v>
       </c>
       <c r="C75" s="2" t="str">
-        <f>RIGHT(A75,4)&amp;B75</f>
+        <f t="shared" si="2"/>
         <v>98442005</v>
       </c>
       <c r="D75" s="9" t="s">
@@ -3201,7 +3204,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="76" spans="1:9">
+    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A76" s="8">
         <v>59096733860</v>
       </c>
@@ -3209,7 +3212,7 @@
         <v>1989</v>
       </c>
       <c r="C76" s="2" t="str">
-        <f>RIGHT(A76,4)&amp;B76</f>
+        <f t="shared" si="2"/>
         <v>38601989</v>
       </c>
       <c r="D76" s="9" t="s">
@@ -3231,7 +3234,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="77" spans="1:9">
+    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A77" s="8">
         <v>50499626842</v>
       </c>
@@ -3239,7 +3242,7 @@
         <v>2000</v>
       </c>
       <c r="C77" s="2" t="str">
-        <f>RIGHT(A77,4)&amp;B77</f>
+        <f t="shared" si="2"/>
         <v>68422000</v>
       </c>
       <c r="D77" s="9" t="s">
@@ -3261,7 +3264,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="78" spans="1:9">
+    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A78" s="8">
         <v>52014422850</v>
       </c>
@@ -3269,7 +3272,7 @@
         <v>2006</v>
       </c>
       <c r="C78" s="2" t="str">
-        <f>RIGHT(A78,4)&amp;B78</f>
+        <f t="shared" si="2"/>
         <v>28502006</v>
       </c>
       <c r="D78" s="9" t="s">
@@ -3291,7 +3294,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="79" spans="1:9">
+    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A79" s="8">
         <v>37446586869</v>
       </c>
@@ -3299,7 +3302,7 @@
         <v>1988</v>
       </c>
       <c r="C79" s="2" t="str">
-        <f>RIGHT(A79,4)&amp;B79</f>
+        <f t="shared" si="2"/>
         <v>68691988</v>
       </c>
       <c r="D79" s="9" t="s">
@@ -3321,7 +3324,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="80" spans="1:9">
+    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A80" s="8">
         <v>42672227896</v>
       </c>
@@ -3329,7 +3332,7 @@
         <v>1995</v>
       </c>
       <c r="C80" s="2" t="str">
-        <f>RIGHT(A80,4)&amp;B80</f>
+        <f t="shared" si="2"/>
         <v>78961995</v>
       </c>
       <c r="D80" s="9" t="s">
@@ -3351,7 +3354,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="81" spans="1:9">
+    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A81" s="8">
         <v>51147754802</v>
       </c>
@@ -3359,7 +3362,7 @@
         <v>2001</v>
       </c>
       <c r="C81" s="2" t="str">
-        <f>RIGHT(A81,4)&amp;B81</f>
+        <f t="shared" si="2"/>
         <v>48022001</v>
       </c>
       <c r="D81" s="9" t="s">
@@ -3381,7 +3384,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="82" spans="1:9">
+    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A82" s="10">
         <v>34606814896</v>
       </c>
@@ -3389,7 +3392,7 @@
         <v>1988</v>
       </c>
       <c r="C82" s="2" t="str">
-        <f>RIGHT(A82,4)&amp;B82</f>
+        <f t="shared" si="2"/>
         <v>48961988</v>
       </c>
       <c r="D82" s="2" t="s">
@@ -3411,7 +3414,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="83" spans="1:9">
+    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A83" s="8">
         <v>47211406810</v>
       </c>
@@ -3419,7 +3422,7 @@
         <v>2003</v>
       </c>
       <c r="C83" s="2" t="str">
-        <f>RIGHT(A83,4)&amp;B83</f>
+        <f t="shared" si="2"/>
         <v>68102003</v>
       </c>
       <c r="D83" s="9" t="s">
@@ -3441,7 +3444,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="84" spans="1:9">
+    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A84" s="8">
         <v>47817611866</v>
       </c>
@@ -3449,7 +3452,7 @@
         <v>1992</v>
       </c>
       <c r="C84" s="2" t="str">
-        <f>RIGHT(A84,4)&amp;B84</f>
+        <f t="shared" si="2"/>
         <v>18661992</v>
       </c>
       <c r="D84" s="9" t="s">
@@ -3471,7 +3474,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="85" spans="1:9">
+    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A85" s="8">
         <v>42202090851</v>
       </c>
@@ -3479,7 +3482,7 @@
         <v>2000</v>
       </c>
       <c r="C85" s="2" t="str">
-        <f>RIGHT(A85,4)&amp;B85</f>
+        <f t="shared" si="2"/>
         <v>08512000</v>
       </c>
       <c r="D85" s="9" t="s">
@@ -3501,7 +3504,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="86" spans="1:9">
+    <row r="86" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A86" s="8">
         <v>52353988822</v>
       </c>
@@ -3509,7 +3512,7 @@
         <v>2003</v>
       </c>
       <c r="C86" s="2" t="str">
-        <f>RIGHT(A86,4)&amp;B86</f>
+        <f t="shared" si="2"/>
         <v>88222003</v>
       </c>
       <c r="D86" s="9" t="s">
@@ -3531,7 +3534,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="87" spans="1:9">
+    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A87" s="8">
         <v>44350770860</v>
       </c>
@@ -3539,7 +3542,7 @@
         <v>2002</v>
       </c>
       <c r="C87" s="2" t="str">
-        <f>RIGHT(A87,4)&amp;B87</f>
+        <f t="shared" si="2"/>
         <v>08602002</v>
       </c>
       <c r="D87" s="9" t="s">
@@ -3561,7 +3564,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="88" spans="1:9">
+    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A88" s="8">
         <v>38011287842</v>
       </c>
@@ -3569,7 +3572,7 @@
         <v>2001</v>
       </c>
       <c r="C88" s="2" t="str">
-        <f>RIGHT(A88,4)&amp;B88</f>
+        <f t="shared" si="2"/>
         <v>78422001</v>
       </c>
       <c r="D88" s="9" t="s">
@@ -3591,7 +3594,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="89" spans="1:9">
+    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A89" s="8">
         <v>8817038342</v>
       </c>
@@ -3599,7 +3602,7 @@
         <v>2004</v>
       </c>
       <c r="C89" s="2" t="str">
-        <f>RIGHT(A89,4)&amp;B89</f>
+        <f t="shared" si="2"/>
         <v>83422004</v>
       </c>
       <c r="D89" s="9" t="s">
@@ -3621,7 +3624,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="90" spans="1:9">
+    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A90" s="8">
         <v>770030475</v>
       </c>
@@ -3629,7 +3632,7 @@
         <v>1979</v>
       </c>
       <c r="C90" s="2" t="str">
-        <f>RIGHT(A90,4)&amp;B90</f>
+        <f t="shared" si="2"/>
         <v>04751979</v>
       </c>
       <c r="D90" s="9" t="s">
@@ -3651,7 +3654,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="91" spans="1:9">
+    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A91" s="8">
         <v>45989936850</v>
       </c>
@@ -3659,7 +3662,7 @@
         <v>1997</v>
       </c>
       <c r="C91" s="2" t="str">
-        <f>RIGHT(A91,4)&amp;B91</f>
+        <f t="shared" si="2"/>
         <v>68501997</v>
       </c>
       <c r="D91" s="9" t="s">
@@ -3681,7 +3684,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="92" spans="1:9">
+    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A92" s="8">
         <v>41460506855</v>
       </c>
@@ -3689,7 +3692,7 @@
         <v>2005</v>
       </c>
       <c r="C92" s="2" t="str">
-        <f>RIGHT(A92,4)&amp;B92</f>
+        <f t="shared" si="2"/>
         <v>68552005</v>
       </c>
       <c r="D92" s="9" t="s">
@@ -3711,7 +3714,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="93" spans="1:9">
+    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A93" s="8">
         <v>47167140805</v>
       </c>
@@ -3719,7 +3722,7 @@
         <v>2000</v>
       </c>
       <c r="C93" s="2" t="str">
-        <f>RIGHT(A93,4)&amp;B93</f>
+        <f t="shared" si="2"/>
         <v>08052000</v>
       </c>
       <c r="D93" s="9" t="s">
@@ -3741,7 +3744,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="94" spans="1:9">
+    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A94" s="8">
         <v>32568233869</v>
       </c>
@@ -3749,7 +3752,7 @@
         <v>1985</v>
       </c>
       <c r="C94" s="2" t="str">
-        <f>RIGHT(A94,4)&amp;B94</f>
+        <f t="shared" si="2"/>
         <v>38691985</v>
       </c>
       <c r="D94" s="9" t="s">
@@ -3771,7 +3774,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="95" spans="1:9">
+    <row r="95" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A95" s="8">
         <v>53833326859</v>
       </c>
@@ -3779,7 +3782,7 @@
         <v>2006</v>
       </c>
       <c r="C95" s="2" t="str">
-        <f>RIGHT(A95,4)&amp;B95</f>
+        <f t="shared" si="2"/>
         <v>68592006</v>
       </c>
       <c r="D95" s="9" t="s">
@@ -3801,7 +3804,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="96" spans="1:9">
+    <row r="96" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A96" s="8">
         <v>52172623890</v>
       </c>
@@ -3809,7 +3812,7 @@
         <v>2005</v>
       </c>
       <c r="C96" s="2" t="str">
-        <f>RIGHT(A96,4)&amp;B96</f>
+        <f t="shared" si="2"/>
         <v>38902005</v>
       </c>
       <c r="D96" s="9" t="s">
@@ -3831,7 +3834,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="97" spans="1:9">
+    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A97" s="8">
         <v>34884914805</v>
       </c>
@@ -3839,7 +3842,7 @@
         <v>1985</v>
       </c>
       <c r="C97" s="2" t="str">
-        <f>RIGHT(A97,4)&amp;B97</f>
+        <f t="shared" si="2"/>
         <v>48051985</v>
       </c>
       <c r="D97" s="9" t="s">
@@ -3861,7 +3864,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="98" spans="1:9">
+    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A98" s="8">
         <v>41755663846</v>
       </c>
@@ -3869,7 +3872,7 @@
         <v>2002</v>
       </c>
       <c r="C98" s="2" t="str">
-        <f>RIGHT(A98,4)&amp;B98</f>
+        <f t="shared" ref="C98:C129" si="3">RIGHT(A98,4)&amp;B98</f>
         <v>38462002</v>
       </c>
       <c r="D98" s="9" t="s">
@@ -3891,7 +3894,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="99" spans="1:9">
+    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A99" s="8">
         <v>42222464846</v>
       </c>
@@ -3899,7 +3902,7 @@
         <v>1994</v>
       </c>
       <c r="C99" s="2" t="str">
-        <f>RIGHT(A99,4)&amp;B99</f>
+        <f t="shared" si="3"/>
         <v>48461994</v>
       </c>
       <c r="D99" s="9" t="s">
@@ -3921,7 +3924,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="100" spans="1:9">
+    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A100" s="8">
         <v>57536852851</v>
       </c>
@@ -3929,7 +3932,7 @@
         <v>2008</v>
       </c>
       <c r="C100" s="2" t="str">
-        <f>RIGHT(A100,4)&amp;B100</f>
+        <f t="shared" si="3"/>
         <v>28512008</v>
       </c>
       <c r="D100" s="9" t="s">
@@ -3951,7 +3954,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="101" spans="1:9">
+    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A101" s="8">
         <v>48556621864</v>
       </c>
@@ -3959,7 +3962,7 @@
         <v>2000</v>
       </c>
       <c r="C101" s="2" t="str">
-        <f>RIGHT(A101,4)&amp;B101</f>
+        <f t="shared" si="3"/>
         <v>18642000</v>
       </c>
       <c r="D101" s="9" t="s">
@@ -3981,7 +3984,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="102" spans="1:9">
+    <row r="102" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A102" s="8">
         <v>50308043820</v>
       </c>
@@ -3989,7 +3992,7 @@
         <v>2001</v>
       </c>
       <c r="C102" s="2" t="str">
-        <f>RIGHT(A102,4)&amp;B102</f>
+        <f t="shared" si="3"/>
         <v>38202001</v>
       </c>
       <c r="D102" s="9" t="s">
@@ -4011,7 +4014,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="103" spans="1:9">
+    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A103" s="8">
         <v>45279130850</v>
       </c>
@@ -4019,7 +4022,7 @@
         <v>2003</v>
       </c>
       <c r="C103" s="2" t="str">
-        <f>RIGHT(A103,4)&amp;B103</f>
+        <f t="shared" si="3"/>
         <v>08502003</v>
       </c>
       <c r="D103" s="9" t="s">
@@ -4041,7 +4044,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="104" spans="1:9">
+    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A104" s="8">
         <v>49190532821</v>
       </c>
@@ -4049,7 +4052,7 @@
         <v>2003</v>
       </c>
       <c r="C104" s="2" t="str">
-        <f>RIGHT(A104,4)&amp;B104</f>
+        <f t="shared" si="3"/>
         <v>28212003</v>
       </c>
       <c r="D104" s="9" t="s">
@@ -4071,7 +4074,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="105" spans="1:9">
+    <row r="105" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A105" s="8">
         <v>53864652871</v>
       </c>
@@ -4079,7 +4082,7 @@
         <v>2006</v>
       </c>
       <c r="C105" s="2" t="str">
-        <f>RIGHT(A105,4)&amp;B105</f>
+        <f t="shared" si="3"/>
         <v>28712006</v>
       </c>
       <c r="D105" s="9" t="s">
@@ -4101,7 +4104,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="106" spans="1:9">
+    <row r="106" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A106" s="8">
         <v>52587009847</v>
       </c>
@@ -4109,7 +4112,7 @@
         <v>2004</v>
       </c>
       <c r="C106" s="2" t="str">
-        <f>RIGHT(A106,4)&amp;B106</f>
+        <f t="shared" si="3"/>
         <v>98472004</v>
       </c>
       <c r="D106" s="9" t="s">
@@ -4131,7 +4134,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="107" spans="1:9">
+    <row r="107" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A107" s="8">
         <v>29911349845</v>
       </c>
@@ -4139,7 +4142,7 @@
         <v>1981</v>
       </c>
       <c r="C107" s="2" t="str">
-        <f>RIGHT(A107,4)&amp;B107</f>
+        <f t="shared" si="3"/>
         <v>98451981</v>
       </c>
       <c r="D107" s="9" t="s">
@@ -4161,7 +4164,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="108" spans="1:9">
+    <row r="108" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A108" s="8">
         <v>52970856832</v>
       </c>
@@ -4169,7 +4172,7 @@
         <v>2001</v>
       </c>
       <c r="C108" s="2" t="str">
-        <f>RIGHT(A108,4)&amp;B108</f>
+        <f t="shared" si="3"/>
         <v>68322001</v>
       </c>
       <c r="D108" s="9" t="s">
@@ -4191,7 +4194,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="109" spans="1:9">
+    <row r="109" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A109" s="8">
         <v>33020819873</v>
       </c>
@@ -4199,7 +4202,7 @@
         <v>1985</v>
       </c>
       <c r="C109" s="2" t="str">
-        <f>RIGHT(A109,4)&amp;B109</f>
+        <f t="shared" si="3"/>
         <v>98731985</v>
       </c>
       <c r="D109" s="9" t="s">
@@ -4221,7 +4224,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="110" spans="1:9">
+    <row r="110" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A110" s="8">
         <v>33091270874</v>
       </c>
@@ -4229,7 +4232,7 @@
         <v>1986</v>
       </c>
       <c r="C110" s="2" t="str">
-        <f>RIGHT(A110,4)&amp;B110</f>
+        <f t="shared" si="3"/>
         <v>08741986</v>
       </c>
       <c r="D110" s="9" t="s">
@@ -4251,7 +4254,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="111" spans="1:9">
+    <row r="111" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A111" s="8">
         <v>27378843814</v>
       </c>
@@ -4259,7 +4262,7 @@
         <v>1977</v>
       </c>
       <c r="C111" s="2" t="str">
-        <f>RIGHT(A111,4)&amp;B111</f>
+        <f t="shared" si="3"/>
         <v>38141977</v>
       </c>
       <c r="D111" s="9" t="s">
@@ -4281,7 +4284,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="112" spans="1:9">
+    <row r="112" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A112" s="8">
         <v>40165009829</v>
       </c>
@@ -4289,7 +4292,7 @@
         <v>2007</v>
       </c>
       <c r="C112" s="2" t="str">
-        <f>RIGHT(A112,4)&amp;B112</f>
+        <f t="shared" si="3"/>
         <v>98292007</v>
       </c>
       <c r="D112" s="9" t="s">
@@ -4311,7 +4314,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="113" spans="1:9">
+    <row r="113" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A113" s="8">
         <v>29170771820</v>
       </c>
@@ -4319,7 +4322,7 @@
         <v>1982</v>
       </c>
       <c r="C113" s="2" t="str">
-        <f>RIGHT(A113,4)&amp;B113</f>
+        <f t="shared" si="3"/>
         <v>18201982</v>
       </c>
       <c r="D113" s="9" t="s">
@@ -4341,7 +4344,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="114" spans="1:9">
+    <row r="114" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A114" s="8">
         <v>25516190843</v>
       </c>
@@ -4349,7 +4352,7 @@
         <v>1975</v>
       </c>
       <c r="C114" s="2" t="str">
-        <f>RIGHT(A114,4)&amp;B114</f>
+        <f t="shared" si="3"/>
         <v>08431975</v>
       </c>
       <c r="D114" s="9" t="s">
@@ -4371,7 +4374,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="115" spans="1:9">
+    <row r="115" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A115" s="8">
         <v>26192473811</v>
       </c>
@@ -4379,7 +4382,7 @@
         <v>1977</v>
       </c>
       <c r="C115" s="2" t="str">
-        <f>RIGHT(A115,4)&amp;B115</f>
+        <f t="shared" si="3"/>
         <v>38111977</v>
       </c>
       <c r="D115" s="9" t="s">
@@ -4401,7 +4404,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="116" spans="1:9">
+    <row r="116" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A116" s="8">
         <v>36322128809</v>
       </c>
@@ -4409,7 +4412,7 @@
         <v>1990</v>
       </c>
       <c r="C116" s="2" t="str">
-        <f>RIGHT(A116,4)&amp;B116</f>
+        <f t="shared" si="3"/>
         <v>88091990</v>
       </c>
       <c r="D116" s="9" t="s">
@@ -4431,7 +4434,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="117" spans="1:9">
+    <row r="117" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A117" s="8">
         <v>28469113801</v>
       </c>
@@ -4439,7 +4442,7 @@
         <v>1980</v>
       </c>
       <c r="C117" s="2" t="str">
-        <f>RIGHT(A117,4)&amp;B117</f>
+        <f t="shared" si="3"/>
         <v>38011980</v>
       </c>
       <c r="D117" s="9" t="s">
@@ -4461,7 +4464,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="118" spans="1:9">
+    <row r="118" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A118" s="8">
         <v>31014693845</v>
       </c>
@@ -4469,7 +4472,7 @@
         <v>1984</v>
       </c>
       <c r="C118" s="2" t="str">
-        <f>RIGHT(A118,4)&amp;B118</f>
+        <f t="shared" si="3"/>
         <v>38451984</v>
       </c>
       <c r="D118" s="9" t="s">
@@ -4491,7 +4494,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="119" spans="1:9">
+    <row r="119" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A119" s="8">
         <v>33887811844</v>
       </c>
@@ -4499,7 +4502,7 @@
         <v>1984</v>
       </c>
       <c r="C119" s="2" t="str">
-        <f>RIGHT(A119,4)&amp;B119</f>
+        <f t="shared" si="3"/>
         <v>18441984</v>
       </c>
       <c r="D119" s="9" t="s">
@@ -4521,7 +4524,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="120" spans="1:9">
+    <row r="120" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A120" s="8">
         <v>28505783808</v>
       </c>
@@ -4529,7 +4532,7 @@
         <v>1980</v>
       </c>
       <c r="C120" s="2" t="str">
-        <f>RIGHT(A120,4)&amp;B120</f>
+        <f t="shared" si="3"/>
         <v>38081980</v>
       </c>
       <c r="D120" s="9" t="s">
@@ -4551,7 +4554,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="121" spans="1:9">
+    <row r="121" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A121" s="1" t="s">
         <v>135</v>
       </c>
@@ -4559,7 +4562,7 @@
         <v>1960</v>
       </c>
       <c r="C121" s="2" t="str">
-        <f>RIGHT(A121,4)&amp;B121</f>
+        <f t="shared" si="3"/>
         <v>78051960</v>
       </c>
       <c r="D121" s="2" t="s">
@@ -4581,7 +4584,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="122" spans="1:9">
+    <row r="122" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A122" s="8">
         <v>48060547801</v>
       </c>
@@ -4589,7 +4592,7 @@
         <v>1997</v>
       </c>
       <c r="C122" s="2" t="str">
-        <f>RIGHT(A122,4)&amp;B122</f>
+        <f t="shared" si="3"/>
         <v>78011997</v>
       </c>
       <c r="D122" s="9" t="s">
@@ -4611,7 +4614,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="123" spans="1:9">
+    <row r="123" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A123" s="8">
         <v>26687173880</v>
       </c>
@@ -4619,7 +4622,7 @@
         <v>1975</v>
       </c>
       <c r="C123" s="2" t="str">
-        <f>RIGHT(A123,4)&amp;B123</f>
+        <f t="shared" si="3"/>
         <v>38801975</v>
       </c>
       <c r="D123" s="9" t="s">
@@ -4641,7 +4644,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="124" spans="1:9">
+    <row r="124" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A124" s="8">
         <v>44610167816</v>
       </c>
@@ -4649,7 +4652,7 @@
         <v>1995</v>
       </c>
       <c r="C124" s="2" t="str">
-        <f>RIGHT(A124,4)&amp;B124</f>
+        <f t="shared" si="3"/>
         <v>78161995</v>
       </c>
       <c r="D124" s="9" t="s">
@@ -4671,7 +4674,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="125" spans="1:9">
+    <row r="125" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A125" s="8">
         <v>37196678800</v>
       </c>
@@ -4679,7 +4682,7 @@
         <v>1989</v>
       </c>
       <c r="C125" s="2" t="str">
-        <f>RIGHT(A125,4)&amp;B125</f>
+        <f t="shared" si="3"/>
         <v>88001989</v>
       </c>
       <c r="D125" s="9" t="s">
@@ -4701,7 +4704,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="126" spans="1:9">
+    <row r="126" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A126" s="8">
         <v>34294701889</v>
       </c>
@@ -4709,7 +4712,7 @@
         <v>1986</v>
       </c>
       <c r="C126" s="2" t="str">
-        <f>RIGHT(A126,4)&amp;B126</f>
+        <f t="shared" si="3"/>
         <v>18891986</v>
       </c>
       <c r="D126" s="9" t="s">
@@ -4731,7 +4734,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="127" spans="1:9">
+    <row r="127" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A127" s="8">
         <v>50400969840</v>
       </c>
@@ -4739,7 +4742,7 @@
         <v>2002</v>
       </c>
       <c r="C127" s="2" t="str">
-        <f>RIGHT(A127,4)&amp;B127</f>
+        <f t="shared" si="3"/>
         <v>98402002</v>
       </c>
       <c r="D127" s="9" t="s">
@@ -4761,7 +4764,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="128" spans="1:9">
+    <row r="128" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A128" s="8">
         <v>39724385833</v>
       </c>
@@ -4769,7 +4772,7 @@
         <v>1991</v>
       </c>
       <c r="C128" s="2" t="str">
-        <f>RIGHT(A128,4)&amp;B128</f>
+        <f t="shared" si="3"/>
         <v>58331991</v>
       </c>
       <c r="D128" s="9" t="s">
@@ -4791,7 +4794,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="129" spans="1:9">
+    <row r="129" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A129" s="8">
         <v>20053874870</v>
       </c>
@@ -4799,7 +4802,7 @@
         <v>1976</v>
       </c>
       <c r="C129" s="2" t="str">
-        <f>RIGHT(A129,4)&amp;B129</f>
+        <f t="shared" si="3"/>
         <v>48701976</v>
       </c>
       <c r="D129" s="9" t="s">
@@ -4821,7 +4824,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="130" spans="1:9">
+    <row r="130" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A130" s="15">
         <v>40542592860</v>
       </c>
@@ -4829,7 +4832,7 @@
         <v>1992</v>
       </c>
       <c r="C130" s="12" t="str">
-        <f>RIGHT(A130,4)&amp;B130</f>
+        <f t="shared" ref="C130:C161" si="4">RIGHT(A130,4)&amp;B130</f>
         <v>28601992</v>
       </c>
       <c r="D130" s="16" t="s">
@@ -4851,7 +4854,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="131" spans="1:9">
+    <row r="131" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A131" s="8">
         <v>48963889840</v>
       </c>
@@ -4859,7 +4862,7 @@
         <v>2000</v>
       </c>
       <c r="C131" s="2" t="str">
-        <f>RIGHT(A131,4)&amp;B131</f>
+        <f t="shared" si="4"/>
         <v>98402000</v>
       </c>
       <c r="D131" s="9" t="s">
@@ -4881,7 +4884,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="132" spans="1:9">
+    <row r="132" spans="1:9" x14ac:dyDescent="0.35">
       <c r="A132" s="8">
         <v>44273964880</v>
       </c>
@@ -4889,7 +4892,7 @@
         <v>1993</v>
       </c>
       <c r="C132" s="2" t="str">
-        <f>RIGHT(A132,4)&amp;B132</f>
+        <f t="shared" si="4"/>
         <v>48801993</v>
       </c>
       <c r="D132" s="9" t="s">

</xml_diff>

<commit_message>
Atualiza certificados: adiciona prefixo "Treinamento" ao curso e novo registro
Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/assets/Modelo Certificado.xlsx
+++ b/assets/Modelo Certificado.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="24334"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30404"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://atlheticanutrition-my.sharepoint.com/personal/digital_platforms_nutramerica_com_br/Documents/DEV/TOTEN CERTIFICADO/assets/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="14_{855DC049-69AE-459E-A0C6-62EC7BE3C0C0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{747F2F3F-641B-44C3-91C1-626DA8B4C0BA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <workbookProtection workbookAlgorithmName="SHA-512" workbookHashValue="NqJ3wjgx3cR7sVkcjUgjQiZb+1Evdvoja7xCh7UBIlMuCccWPD+KD7gWt7OFG5fGKNERamv/HrY1kCOk7uqHKQ==" workbookSaltValue="QbyEgElAzcOx3LPBthQYDA==" workbookSpinCount="100000" lockStructure="1"/>
   <bookViews>
     <workbookView xWindow="8150" yWindow="2570" windowWidth="28800" windowHeight="15370" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
@@ -35,15 +35,12 @@
         <xcalcf:feature name="microsoft.com:ARRAYTEXT_WF"/>
       </xcalcf:calcFeatures>
     </ext>
-    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
-      <xlwcv:version setVersion="1"/>
-    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="538" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="539" uniqueCount="149">
   <si>
     <t>CPF</t>
   </si>
@@ -75,7 +72,7 @@
     <t>ADRIANA DE LIMA CARVALHO</t>
   </si>
   <si>
-    <t>BOAS PRÁTICAS DE FABRICAÇÃO E SEGURANÇA DOS ALIMENTOS</t>
+    <t>Treinamento BOAS PRÁTICAS DE FABRICAÇÃO E SEGURANÇA DOS ALIMENTOS</t>
   </si>
   <si>
     <t>Agosto</t>
@@ -84,7 +81,7 @@
     <t>1h30</t>
   </si>
   <si>
-    <t>ALBA VALERIA ROSEMBERG CHIOZZINI TESSI</t>
+    <t>ALBA V. ROSEMBERG CHIOZZINI TESSI</t>
   </si>
   <si>
     <t>ALESSANDRO SOUSA DE ALMEIDA</t>
@@ -142,6 +139,9 @@
   </si>
   <si>
     <t>ANGELA MARCIA DE SOUZA MARQUES</t>
+  </si>
+  <si>
+    <t>17541201804</t>
   </si>
   <si>
     <t xml:space="preserve">ANGELICA ALBARICCI DE ANGELIS DE SOUZA </t>
@@ -496,7 +496,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="[$-F400]h:mm:ss\ AM/PM"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="4">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -944,22 +944,22 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <dimension ref="A1:I132"/>
-  <sheetFormatPr defaultColWidth="9.1796875" defaultRowHeight="15.5" x14ac:dyDescent="0.35"/>
+  <sheetFormatPr defaultColWidth="9.140625" defaultRowHeight="15.75"/>
   <cols>
-    <col min="1" max="1" width="16.1796875" style="6" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="19.81640625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="19.7265625" style="3" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="53.453125" style="3" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="67" style="3" customWidth="1"/>
-    <col min="6" max="9" width="9.54296875" style="3" customWidth="1"/>
-    <col min="10" max="14" width="9.1796875" style="3"/>
-    <col min="15" max="15" width="34.1796875" style="3" bestFit="1" customWidth="1"/>
-    <col min="16" max="16" width="34.1796875" style="3" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" style="6" hidden="1" customWidth="1"/>
+    <col min="2" max="2" width="19.85546875" style="3" hidden="1" customWidth="1"/>
+    <col min="3" max="3" width="19.7109375" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="53.42578125" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="84.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="6" max="9" width="9.5703125" style="3" customWidth="1"/>
+    <col min="10" max="14" width="9.140625" style="3"/>
+    <col min="15" max="15" width="34.140625" style="3" bestFit="1" customWidth="1"/>
+    <col min="16" max="16" width="34.140625" style="3" customWidth="1"/>
     <col min="17" max="17" width="37" style="3" bestFit="1" customWidth="1"/>
-    <col min="18" max="16384" width="9.1796875" style="3"/>
+    <col min="18" max="16384" width="9.140625" style="3"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="1" spans="1:9">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -988,7 +988,7 @@
         <v>8</v>
       </c>
     </row>
-    <row r="2" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="2" spans="1:9">
       <c r="A2" s="8">
         <v>4349484469</v>
       </c>
@@ -996,7 +996,7 @@
         <v>1981</v>
       </c>
       <c r="C2" s="2" t="str">
-        <f t="shared" ref="C2:C33" si="0">RIGHT(A2,4)&amp;B2</f>
+        <f>RIGHT(A2,4)&amp;B2</f>
         <v>44691981</v>
       </c>
       <c r="D2" s="9" t="s">
@@ -1018,7 +1018,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="3" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="3" spans="1:9">
       <c r="A3" s="8">
         <v>27672701878</v>
       </c>
@@ -1026,7 +1026,7 @@
         <v>1979</v>
       </c>
       <c r="C3" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A3,4)&amp;B3</f>
         <v>18781979</v>
       </c>
       <c r="D3" s="9" t="s">
@@ -1048,7 +1048,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="4" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="4" spans="1:9">
       <c r="A4" s="8">
         <v>35353327888</v>
       </c>
@@ -1056,7 +1056,7 @@
         <v>1987</v>
       </c>
       <c r="C4" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A4,4)&amp;B4</f>
         <v>78881987</v>
       </c>
       <c r="D4" s="9" t="s">
@@ -1078,7 +1078,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="5" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="5" spans="1:9">
       <c r="A5" s="8">
         <v>41197627855</v>
       </c>
@@ -1086,7 +1086,7 @@
         <v>1992</v>
       </c>
       <c r="C5" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A5,4)&amp;B5</f>
         <v>78551992</v>
       </c>
       <c r="D5" s="9" t="s">
@@ -1108,7 +1108,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="6" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="6" spans="1:9">
       <c r="A6" s="8">
         <v>53994007828</v>
       </c>
@@ -1116,7 +1116,7 @@
         <v>2005</v>
       </c>
       <c r="C6" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A6,4)&amp;B6</f>
         <v>78282005</v>
       </c>
       <c r="D6" s="9" t="s">
@@ -1138,7 +1138,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="7" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="7" spans="1:9">
       <c r="A7" s="8">
         <v>43876868807</v>
       </c>
@@ -1146,7 +1146,7 @@
         <v>1996</v>
       </c>
       <c r="C7" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A7,4)&amp;B7</f>
         <v>88071996</v>
       </c>
       <c r="D7" s="9" t="s">
@@ -1168,7 +1168,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="8" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="8" spans="1:9">
       <c r="A8" s="10">
         <v>42186704803</v>
       </c>
@@ -1176,7 +1176,7 @@
         <v>1996</v>
       </c>
       <c r="C8" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A8,4)&amp;B8</f>
         <v>48031996</v>
       </c>
       <c r="D8" s="2" t="s">
@@ -1198,7 +1198,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="9" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="9" spans="1:9">
       <c r="A9" s="1" t="s">
         <v>19</v>
       </c>
@@ -1206,7 +1206,7 @@
         <v>1997</v>
       </c>
       <c r="C9" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A9,4)&amp;B9</f>
         <v>58801997</v>
       </c>
       <c r="D9" s="2" t="s">
@@ -1228,7 +1228,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="10" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="10" spans="1:9">
       <c r="A10" s="8">
         <v>44666032860</v>
       </c>
@@ -1236,7 +1236,7 @@
         <v>1994</v>
       </c>
       <c r="C10" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A10,4)&amp;B10</f>
         <v>28601994</v>
       </c>
       <c r="D10" s="9" t="s">
@@ -1258,7 +1258,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="11" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="11" spans="1:9">
       <c r="A11" s="8">
         <v>46967903802</v>
       </c>
@@ -1266,7 +1266,7 @@
         <v>2007</v>
       </c>
       <c r="C11" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A11,4)&amp;B11</f>
         <v>38022007</v>
       </c>
       <c r="D11" s="9" t="s">
@@ -1288,7 +1288,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="12" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="12" spans="1:9">
       <c r="A12" s="8">
         <v>47193017896</v>
       </c>
@@ -1296,7 +1296,7 @@
         <v>2000</v>
       </c>
       <c r="C12" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A12,4)&amp;B12</f>
         <v>78962000</v>
       </c>
       <c r="D12" s="9" t="s">
@@ -1318,7 +1318,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="13" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="13" spans="1:9">
       <c r="A13" s="8">
         <v>34687383823</v>
       </c>
@@ -1326,7 +1326,7 @@
         <v>2001</v>
       </c>
       <c r="C13" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A13,4)&amp;B13</f>
         <v>38232001</v>
       </c>
       <c r="D13" s="9" t="s">
@@ -1348,7 +1348,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="14" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="14" spans="1:9">
       <c r="A14" s="8">
         <v>37835487802</v>
       </c>
@@ -1356,7 +1356,7 @@
         <v>1987</v>
       </c>
       <c r="C14" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A14,4)&amp;B14</f>
         <v>78021987</v>
       </c>
       <c r="D14" s="9" t="s">
@@ -1378,7 +1378,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="15" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="15" spans="1:9">
       <c r="A15" s="7" t="s">
         <v>26</v>
       </c>
@@ -1386,7 +1386,7 @@
         <v>1982</v>
       </c>
       <c r="C15" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A15,4)&amp;B15</f>
         <v>97841982</v>
       </c>
       <c r="D15" s="5" t="s">
@@ -1408,7 +1408,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="16" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="16" spans="1:9">
       <c r="A16" s="8">
         <v>48954491812</v>
       </c>
@@ -1416,7 +1416,7 @@
         <v>1997</v>
       </c>
       <c r="C16" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A16,4)&amp;B16</f>
         <v>18121997</v>
       </c>
       <c r="D16" s="9" t="s">
@@ -1438,7 +1438,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="17" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="17" spans="1:9">
       <c r="A17" s="8">
         <v>46997604811</v>
       </c>
@@ -1446,7 +1446,7 @@
         <v>1995</v>
       </c>
       <c r="C17" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A17,4)&amp;B17</f>
         <v>48111995</v>
       </c>
       <c r="D17" s="9" t="s">
@@ -1468,7 +1468,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="18" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="18" spans="1:9">
       <c r="A18" s="8">
         <v>36945656802</v>
       </c>
@@ -1476,7 +1476,7 @@
         <v>1988</v>
       </c>
       <c r="C18" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A18,4)&amp;B18</f>
         <v>68021988</v>
       </c>
       <c r="D18" s="9" t="s">
@@ -1498,7 +1498,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="19" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="19" spans="1:9">
       <c r="A19" s="10">
         <v>26920249820</v>
       </c>
@@ -1506,7 +1506,7 @@
         <v>1979</v>
       </c>
       <c r="C19" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A19,4)&amp;B19</f>
         <v>98201979</v>
       </c>
       <c r="D19" s="5" t="s">
@@ -1528,7 +1528,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="20" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="20" spans="1:9">
       <c r="A20" s="8">
         <v>25495474899</v>
       </c>
@@ -1536,7 +1536,7 @@
         <v>1971</v>
       </c>
       <c r="C20" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A20,4)&amp;B20</f>
         <v>48991971</v>
       </c>
       <c r="D20" s="9" t="s">
@@ -1558,15 +1558,19 @@
         <v>12</v>
       </c>
     </row>
-    <row r="21" spans="1:9" x14ac:dyDescent="0.35">
-      <c r="A21" s="1"/>
-      <c r="B21" s="2"/>
+    <row r="21" spans="1:9">
+      <c r="A21" s="1" t="s">
+        <v>33</v>
+      </c>
+      <c r="B21" s="2">
+        <v>1973</v>
+      </c>
       <c r="C21" s="2" t="str">
-        <f t="shared" si="0"/>
-        <v/>
+        <f>RIGHT(A21,4)&amp;B21</f>
+        <v>18041973</v>
       </c>
       <c r="D21" s="2" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="E21" s="2" t="s">
         <v>10</v>
@@ -1584,7 +1588,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="22" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="22" spans="1:9">
       <c r="A22" s="8">
         <v>31230944800</v>
       </c>
@@ -1592,11 +1596,11 @@
         <v>1977</v>
       </c>
       <c r="C22" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A22,4)&amp;B22</f>
         <v>48001977</v>
       </c>
       <c r="D22" s="9" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="E22" s="2" t="s">
         <v>10</v>
@@ -1614,7 +1618,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="23" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="23" spans="1:9">
       <c r="A23" s="8">
         <v>50155292870</v>
       </c>
@@ -1622,11 +1626,11 @@
         <v>2000</v>
       </c>
       <c r="C23" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A23,4)&amp;B23</f>
         <v>28702000</v>
       </c>
       <c r="D23" s="9" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="E23" s="2" t="s">
         <v>10</v>
@@ -1644,7 +1648,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="24" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="24" spans="1:9">
       <c r="A24" s="8">
         <v>46476927876</v>
       </c>
@@ -1652,11 +1656,11 @@
         <v>1996</v>
       </c>
       <c r="C24" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A24,4)&amp;B24</f>
         <v>78761996</v>
       </c>
       <c r="D24" s="9" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="E24" s="2" t="s">
         <v>10</v>
@@ -1674,7 +1678,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="25" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="25" spans="1:9">
       <c r="A25" s="8">
         <v>42039343890</v>
       </c>
@@ -1682,11 +1686,11 @@
         <v>1993</v>
       </c>
       <c r="C25" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A25,4)&amp;B25</f>
         <v>38901993</v>
       </c>
       <c r="D25" s="9" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="E25" s="2" t="s">
         <v>10</v>
@@ -1704,7 +1708,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="26" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="26" spans="1:9">
       <c r="A26" s="8">
         <v>44891522801</v>
       </c>
@@ -1712,11 +1716,11 @@
         <v>1996</v>
       </c>
       <c r="C26" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A26,4)&amp;B26</f>
         <v>28011996</v>
       </c>
       <c r="D26" s="9" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="E26" s="2" t="s">
         <v>10</v>
@@ -1734,7 +1738,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="27" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="27" spans="1:9">
       <c r="A27" s="8">
         <v>36377720866</v>
       </c>
@@ -1742,11 +1746,11 @@
         <v>1992</v>
       </c>
       <c r="C27" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A27,4)&amp;B27</f>
         <v>08661992</v>
       </c>
       <c r="D27" s="9" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="E27" s="2" t="s">
         <v>10</v>
@@ -1764,7 +1768,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="28" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="28" spans="1:9">
       <c r="A28" s="8">
         <v>52750031885</v>
       </c>
@@ -1772,11 +1776,11 @@
         <v>2003</v>
       </c>
       <c r="C28" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A28,4)&amp;B28</f>
         <v>18852003</v>
       </c>
       <c r="D28" s="9" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="E28" s="2" t="s">
         <v>10</v>
@@ -1794,7 +1798,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="29" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="29" spans="1:9">
       <c r="A29" s="11">
         <v>39974249856</v>
       </c>
@@ -1802,11 +1806,11 @@
         <v>1991</v>
       </c>
       <c r="C29" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A29,4)&amp;B29</f>
         <v>98561991</v>
       </c>
       <c r="D29" s="2" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="E29" s="2" t="s">
         <v>10</v>
@@ -1824,7 +1828,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="30" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="30" spans="1:9">
       <c r="A30" s="8">
         <v>37714454857</v>
       </c>
@@ -1832,11 +1836,11 @@
         <v>1995</v>
       </c>
       <c r="C30" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A30,4)&amp;B30</f>
         <v>48571995</v>
       </c>
       <c r="D30" s="9" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="E30" s="2" t="s">
         <v>10</v>
@@ -1854,7 +1858,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="31" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="31" spans="1:9">
       <c r="A31" s="8">
         <v>37606164886</v>
       </c>
@@ -1862,11 +1866,11 @@
         <v>1995</v>
       </c>
       <c r="C31" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A31,4)&amp;B31</f>
         <v>48861995</v>
       </c>
       <c r="D31" s="9" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="E31" s="2" t="s">
         <v>10</v>
@@ -1884,7 +1888,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="32" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="32" spans="1:9">
       <c r="A32" s="8">
         <v>33864275881</v>
       </c>
@@ -1892,11 +1896,11 @@
         <v>1982</v>
       </c>
       <c r="C32" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A32,4)&amp;B32</f>
         <v>58811982</v>
       </c>
       <c r="D32" s="9" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="E32" s="2" t="s">
         <v>10</v>
@@ -1914,7 +1918,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="33" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="33" spans="1:9">
       <c r="A33" s="8">
         <v>35971031899</v>
       </c>
@@ -1922,11 +1926,11 @@
         <v>1988</v>
       </c>
       <c r="C33" s="2" t="str">
-        <f t="shared" si="0"/>
+        <f>RIGHT(A33,4)&amp;B33</f>
         <v>18991988</v>
       </c>
       <c r="D33" s="9" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="E33" s="2" t="s">
         <v>10</v>
@@ -1944,7 +1948,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="34" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="34" spans="1:9">
       <c r="A34" s="8">
         <v>37383312805</v>
       </c>
@@ -1952,11 +1956,11 @@
         <v>1987</v>
       </c>
       <c r="C34" s="2" t="str">
-        <f t="shared" ref="C34:C65" si="1">RIGHT(A34,4)&amp;B34</f>
+        <f>RIGHT(A34,4)&amp;B34</f>
         <v>28051987</v>
       </c>
       <c r="D34" s="9" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="E34" s="2" t="s">
         <v>10</v>
@@ -1974,19 +1978,19 @@
         <v>12</v>
       </c>
     </row>
-    <row r="35" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="35" spans="1:9">
       <c r="A35" s="8">
-        <v>35989473800</v>
+        <v>47128318801</v>
       </c>
       <c r="B35" s="9">
         <v>2002</v>
       </c>
       <c r="C35" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>38002002</v>
+        <f>RIGHT(A35,4)&amp;B35</f>
+        <v>88012002</v>
       </c>
       <c r="D35" s="9" t="s">
-        <v>47</v>
+        <v>48</v>
       </c>
       <c r="E35" s="2" t="s">
         <v>10</v>
@@ -2004,19 +2008,19 @@
         <v>12</v>
       </c>
     </row>
-    <row r="36" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="36" spans="1:9">
       <c r="A36" s="8">
-        <v>47128318801</v>
+        <v>35989473800</v>
       </c>
       <c r="B36" s="9">
         <v>1987</v>
       </c>
       <c r="C36" s="2" t="str">
-        <f t="shared" si="1"/>
-        <v>88011987</v>
+        <f>RIGHT(A36,4)&amp;B36</f>
+        <v>38001987</v>
       </c>
       <c r="D36" s="9" t="s">
-        <v>48</v>
+        <v>49</v>
       </c>
       <c r="E36" s="2" t="s">
         <v>10</v>
@@ -2034,7 +2038,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="37" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="37" spans="1:9">
       <c r="A37" s="8">
         <v>53700882840</v>
       </c>
@@ -2042,11 +2046,11 @@
         <v>2007</v>
       </c>
       <c r="C37" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A37,4)&amp;B37</f>
         <v>28402007</v>
       </c>
       <c r="D37" s="9" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="E37" s="2" t="s">
         <v>10</v>
@@ -2064,7 +2068,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="38" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="38" spans="1:9">
       <c r="A38" s="8">
         <v>43736502842</v>
       </c>
@@ -2072,11 +2076,11 @@
         <v>1992</v>
       </c>
       <c r="C38" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A38,4)&amp;B38</f>
         <v>28421992</v>
       </c>
       <c r="D38" s="9" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="E38" s="2" t="s">
         <v>10</v>
@@ -2094,7 +2098,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="39" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="39" spans="1:9">
       <c r="A39" s="8">
         <v>45884235844</v>
       </c>
@@ -2102,11 +2106,11 @@
         <v>1996</v>
       </c>
       <c r="C39" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A39,4)&amp;B39</f>
         <v>58441996</v>
       </c>
       <c r="D39" s="9" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="E39" s="2" t="s">
         <v>10</v>
@@ -2124,7 +2128,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="40" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="40" spans="1:9">
       <c r="A40" s="8">
         <v>44020167893</v>
       </c>
@@ -2132,11 +2136,11 @@
         <v>1996</v>
       </c>
       <c r="C40" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A40,4)&amp;B40</f>
         <v>78931996</v>
       </c>
       <c r="D40" s="9" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="E40" s="2" t="s">
         <v>10</v>
@@ -2154,7 +2158,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="41" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="41" spans="1:9">
       <c r="A41" s="8">
         <v>33434644814</v>
       </c>
@@ -2162,11 +2166,11 @@
         <v>1985</v>
       </c>
       <c r="C41" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A41,4)&amp;B41</f>
         <v>48141985</v>
       </c>
       <c r="D41" s="9" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="E41" s="2" t="s">
         <v>10</v>
@@ -2184,7 +2188,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="42" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="42" spans="1:9">
       <c r="A42" s="8">
         <v>43139451806</v>
       </c>
@@ -2192,11 +2196,11 @@
         <v>1995</v>
       </c>
       <c r="C42" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A42,4)&amp;B42</f>
         <v>18061995</v>
       </c>
       <c r="D42" s="9" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="E42" s="2" t="s">
         <v>10</v>
@@ -2214,7 +2218,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="43" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="43" spans="1:9">
       <c r="A43" s="10">
         <v>24944634838</v>
       </c>
@@ -2222,11 +2226,11 @@
         <v>1976</v>
       </c>
       <c r="C43" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A43,4)&amp;B43</f>
         <v>48381976</v>
       </c>
       <c r="D43" s="2" t="s">
-        <v>55</v>
+        <v>56</v>
       </c>
       <c r="E43" s="2" t="s">
         <v>10</v>
@@ -2244,7 +2248,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="44" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="44" spans="1:9">
       <c r="A44" s="8">
         <v>28801880839</v>
       </c>
@@ -2252,11 +2256,11 @@
         <v>1981</v>
       </c>
       <c r="C44" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A44,4)&amp;B44</f>
         <v>08391981</v>
       </c>
       <c r="D44" s="9" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="E44" s="2" t="s">
         <v>10</v>
@@ -2274,7 +2278,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="45" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="45" spans="1:9">
       <c r="A45" s="8">
         <v>41667619861</v>
       </c>
@@ -2282,11 +2286,11 @@
         <v>2003</v>
       </c>
       <c r="C45" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A45,4)&amp;B45</f>
         <v>98612003</v>
       </c>
       <c r="D45" s="9" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="E45" s="2" t="s">
         <v>10</v>
@@ -2304,7 +2308,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="46" spans="1:9">
       <c r="A46" s="8">
         <v>10838890440</v>
       </c>
@@ -2312,11 +2316,11 @@
         <v>1993</v>
       </c>
       <c r="C46" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A46,4)&amp;B46</f>
         <v>04401993</v>
       </c>
       <c r="D46" s="9" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="E46" s="2" t="s">
         <v>10</v>
@@ -2334,7 +2338,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="47" spans="1:9">
       <c r="A47" s="8">
         <v>43118475803</v>
       </c>
@@ -2342,11 +2346,11 @@
         <v>1996</v>
       </c>
       <c r="C47" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A47,4)&amp;B47</f>
         <v>58031996</v>
       </c>
       <c r="D47" s="9" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="E47" s="2" t="s">
         <v>10</v>
@@ -2364,7 +2368,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="48" spans="1:9">
       <c r="A48" s="8">
         <v>47440294858</v>
       </c>
@@ -2372,11 +2376,11 @@
         <v>1998</v>
       </c>
       <c r="C48" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A48,4)&amp;B48</f>
         <v>48581998</v>
       </c>
       <c r="D48" s="9" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="E48" s="2" t="s">
         <v>10</v>
@@ -2394,19 +2398,19 @@
         <v>12</v>
       </c>
     </row>
-    <row r="49" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="49" spans="1:9">
       <c r="A49" s="1" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="B49" s="2">
         <v>1978</v>
       </c>
       <c r="C49" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A49,4)&amp;B49</f>
         <v>08671978</v>
       </c>
       <c r="D49" s="2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="E49" s="2" t="s">
         <v>10</v>
@@ -2424,7 +2428,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="50" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="50" spans="1:9">
       <c r="A50" s="8">
         <v>37257970807</v>
       </c>
@@ -2432,11 +2436,11 @@
         <v>2000</v>
       </c>
       <c r="C50" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A50,4)&amp;B50</f>
         <v>08072000</v>
       </c>
       <c r="D50" s="9" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="E50" s="2" t="s">
         <v>10</v>
@@ -2454,7 +2458,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="51" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="51" spans="1:9">
       <c r="A51" s="8">
         <v>42247533833</v>
       </c>
@@ -2462,11 +2466,11 @@
         <v>1992</v>
       </c>
       <c r="C51" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A51,4)&amp;B51</f>
         <v>38331992</v>
       </c>
       <c r="D51" s="9" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="E51" s="2" t="s">
         <v>10</v>
@@ -2484,7 +2488,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="52" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="52" spans="1:9">
       <c r="A52" s="8">
         <v>45367371892</v>
       </c>
@@ -2492,11 +2496,11 @@
         <v>1995</v>
       </c>
       <c r="C52" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A52,4)&amp;B52</f>
         <v>18921995</v>
       </c>
       <c r="D52" s="9" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="E52" s="2" t="s">
         <v>10</v>
@@ -2514,7 +2518,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="53" spans="1:9">
       <c r="A53" s="8">
         <v>44896404807</v>
       </c>
@@ -2522,11 +2526,11 @@
         <v>2002</v>
       </c>
       <c r="C53" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A53,4)&amp;B53</f>
         <v>48072002</v>
       </c>
       <c r="D53" s="9" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="E53" s="2" t="s">
         <v>10</v>
@@ -2544,7 +2548,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="54" spans="1:9">
       <c r="A54" s="8">
         <v>42659165890</v>
       </c>
@@ -2552,11 +2556,11 @@
         <v>1994</v>
       </c>
       <c r="C54" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A54,4)&amp;B54</f>
         <v>58901994</v>
       </c>
       <c r="D54" s="9" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="E54" s="2" t="s">
         <v>10</v>
@@ -2574,7 +2578,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="55" spans="1:9">
       <c r="A55" s="8">
         <v>36526421806</v>
       </c>
@@ -2582,11 +2586,11 @@
         <v>1987</v>
       </c>
       <c r="C55" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A55,4)&amp;B55</f>
         <v>18061987</v>
       </c>
       <c r="D55" s="9" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="E55" s="2" t="s">
         <v>10</v>
@@ -2604,7 +2608,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="56" spans="1:9">
       <c r="A56" s="8">
         <v>53703468874</v>
       </c>
@@ -2612,11 +2616,11 @@
         <v>2006</v>
       </c>
       <c r="C56" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A56,4)&amp;B56</f>
         <v>88742006</v>
       </c>
       <c r="D56" s="9" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="E56" s="2" t="s">
         <v>10</v>
@@ -2634,7 +2638,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="57" spans="1:9">
       <c r="A57" s="8">
         <v>49193907850</v>
       </c>
@@ -2642,11 +2646,11 @@
         <v>2003</v>
       </c>
       <c r="C57" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A57,4)&amp;B57</f>
         <v>78502003</v>
       </c>
       <c r="D57" s="9" t="s">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="E57" s="2" t="s">
         <v>10</v>
@@ -2664,7 +2668,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="58" spans="1:9">
       <c r="A58" s="8">
         <v>51369270895</v>
       </c>
@@ -2672,11 +2676,11 @@
         <v>2003</v>
       </c>
       <c r="C58" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A58,4)&amp;B58</f>
         <v>08952003</v>
       </c>
       <c r="D58" s="9" t="s">
-        <v>71</v>
+        <v>72</v>
       </c>
       <c r="E58" s="2" t="s">
         <v>10</v>
@@ -2694,7 +2698,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="59" spans="1:9">
       <c r="A59" s="8">
         <v>53316429859</v>
       </c>
@@ -2702,11 +2706,11 @@
         <v>2003</v>
       </c>
       <c r="C59" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A59,4)&amp;B59</f>
         <v>98592003</v>
       </c>
       <c r="D59" s="9" t="s">
-        <v>72</v>
+        <v>73</v>
       </c>
       <c r="E59" s="2" t="s">
         <v>10</v>
@@ -2724,7 +2728,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="60" spans="1:9">
       <c r="A60" s="8">
         <v>27953697882</v>
       </c>
@@ -2732,11 +2736,11 @@
         <v>1977</v>
       </c>
       <c r="C60" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A60,4)&amp;B60</f>
         <v>78821977</v>
       </c>
       <c r="D60" s="9" t="s">
-        <v>73</v>
+        <v>74</v>
       </c>
       <c r="E60" s="2" t="s">
         <v>10</v>
@@ -2754,7 +2758,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="61" spans="1:9">
       <c r="A61" s="8">
         <v>50511623801</v>
       </c>
@@ -2762,11 +2766,11 @@
         <v>2008</v>
       </c>
       <c r="C61" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A61,4)&amp;B61</f>
         <v>38012008</v>
       </c>
       <c r="D61" s="17" t="s">
-        <v>74</v>
+        <v>75</v>
       </c>
       <c r="E61" s="2" t="s">
         <v>10</v>
@@ -2784,7 +2788,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="62" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="62" spans="1:9">
       <c r="A62" s="8">
         <v>39984951855</v>
       </c>
@@ -2792,11 +2796,11 @@
         <v>1991</v>
       </c>
       <c r="C62" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A62,4)&amp;B62</f>
         <v>18551991</v>
       </c>
       <c r="D62" s="9" t="s">
-        <v>75</v>
+        <v>76</v>
       </c>
       <c r="E62" s="2" t="s">
         <v>10</v>
@@ -2814,19 +2818,19 @@
         <v>12</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="63" spans="1:9">
       <c r="A63" s="1" t="s">
-        <v>76</v>
+        <v>77</v>
       </c>
       <c r="B63" s="2">
         <v>1990</v>
       </c>
       <c r="C63" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A63,4)&amp;B63</f>
         <v>88071990</v>
       </c>
       <c r="D63" s="14" t="s">
-        <v>77</v>
+        <v>78</v>
       </c>
       <c r="E63" s="2" t="s">
         <v>10</v>
@@ -2844,7 +2848,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="64" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="64" spans="1:9">
       <c r="A64" s="8">
         <v>35440649875</v>
       </c>
@@ -2852,11 +2856,11 @@
         <v>1990</v>
       </c>
       <c r="C64" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A64,4)&amp;B64</f>
         <v>98751990</v>
       </c>
       <c r="D64" s="9" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="E64" s="2" t="s">
         <v>10</v>
@@ -2874,7 +2878,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="65" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="65" spans="1:9">
       <c r="A65" s="14">
         <v>16716444840</v>
       </c>
@@ -2882,11 +2886,11 @@
         <v>1974</v>
       </c>
       <c r="C65" s="2" t="str">
-        <f t="shared" si="1"/>
+        <f>RIGHT(A65,4)&amp;B65</f>
         <v>48401974</v>
       </c>
       <c r="D65" s="14" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="E65" s="2" t="s">
         <v>10</v>
@@ -2904,7 +2908,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="66" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="66" spans="1:9">
       <c r="A66" s="8">
         <v>38214626803</v>
       </c>
@@ -2912,11 +2916,11 @@
         <v>1988</v>
       </c>
       <c r="C66" s="2" t="str">
-        <f t="shared" ref="C66:C97" si="2">RIGHT(A66,4)&amp;B66</f>
+        <f>RIGHT(A66,4)&amp;B66</f>
         <v>68031988</v>
       </c>
       <c r="D66" s="9" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="E66" s="2" t="s">
         <v>10</v>
@@ -2934,7 +2938,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="67" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="67" spans="1:9">
       <c r="A67" s="8">
         <v>57181251805</v>
       </c>
@@ -2942,11 +2946,11 @@
         <v>2004</v>
       </c>
       <c r="C67" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A67,4)&amp;B67</f>
         <v>18052004</v>
       </c>
       <c r="D67" s="9" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="E67" s="2" t="s">
         <v>10</v>
@@ -2964,7 +2968,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="68" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="68" spans="1:9">
       <c r="A68" s="8">
         <v>41634273842</v>
       </c>
@@ -2972,11 +2976,11 @@
         <v>1992</v>
       </c>
       <c r="C68" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A68,4)&amp;B68</f>
         <v>38421992</v>
       </c>
       <c r="D68" s="9" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="E68" s="2" t="s">
         <v>10</v>
@@ -2994,7 +2998,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="69" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="69" spans="1:9">
       <c r="A69" s="10">
         <v>22351070879</v>
       </c>
@@ -3002,11 +3006,11 @@
         <v>1981</v>
       </c>
       <c r="C69" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A69,4)&amp;B69</f>
         <v>08791981</v>
       </c>
       <c r="D69" s="2" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="E69" s="2" t="s">
         <v>10</v>
@@ -3024,7 +3028,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="70" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="70" spans="1:9">
       <c r="A70" s="8">
         <v>25500655817</v>
       </c>
@@ -3032,11 +3036,11 @@
         <v>1977</v>
       </c>
       <c r="C70" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A70,4)&amp;B70</f>
         <v>58171977</v>
       </c>
       <c r="D70" s="9" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="E70" s="2" t="s">
         <v>10</v>
@@ -3054,7 +3058,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="71" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="71" spans="1:9">
       <c r="A71" s="8">
         <v>39869048838</v>
       </c>
@@ -3062,11 +3066,11 @@
         <v>1992</v>
       </c>
       <c r="C71" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A71,4)&amp;B71</f>
         <v>88381992</v>
       </c>
       <c r="D71" s="9" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="E71" s="2" t="s">
         <v>10</v>
@@ -3084,7 +3088,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="72" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="72" spans="1:9">
       <c r="A72" s="8">
         <v>52817337883</v>
       </c>
@@ -3092,11 +3096,11 @@
         <v>2002</v>
       </c>
       <c r="C72" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A72,4)&amp;B72</f>
         <v>78832002</v>
       </c>
       <c r="D72" s="9" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="E72" s="2" t="s">
         <v>10</v>
@@ -3114,7 +3118,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="73" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="73" spans="1:9">
       <c r="A73" s="8">
         <v>16705635886</v>
       </c>
@@ -3122,11 +3126,11 @@
         <v>1976</v>
       </c>
       <c r="C73" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A73,4)&amp;B73</f>
         <v>58861976</v>
       </c>
       <c r="D73" s="9" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="E73" s="2" t="s">
         <v>10</v>
@@ -3144,7 +3148,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="74" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="74" spans="1:9">
       <c r="A74" s="8">
         <v>52614291889</v>
       </c>
@@ -3152,11 +3156,11 @@
         <v>2005</v>
       </c>
       <c r="C74" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A74,4)&amp;B74</f>
         <v>18892005</v>
       </c>
       <c r="D74" s="9" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="E74" s="2" t="s">
         <v>10</v>
@@ -3174,7 +3178,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="75" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="75" spans="1:9">
       <c r="A75" s="8">
         <v>37241029844</v>
       </c>
@@ -3182,11 +3186,11 @@
         <v>2005</v>
       </c>
       <c r="C75" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A75,4)&amp;B75</f>
         <v>98442005</v>
       </c>
       <c r="D75" s="9" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="E75" s="2" t="s">
         <v>10</v>
@@ -3204,7 +3208,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="76" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="76" spans="1:9">
       <c r="A76" s="8">
         <v>59096733860</v>
       </c>
@@ -3212,11 +3216,11 @@
         <v>1989</v>
       </c>
       <c r="C76" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A76,4)&amp;B76</f>
         <v>38601989</v>
       </c>
       <c r="D76" s="9" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="E76" s="2" t="s">
         <v>10</v>
@@ -3234,7 +3238,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="77" spans="1:9">
       <c r="A77" s="8">
         <v>50499626842</v>
       </c>
@@ -3242,11 +3246,11 @@
         <v>2000</v>
       </c>
       <c r="C77" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A77,4)&amp;B77</f>
         <v>68422000</v>
       </c>
       <c r="D77" s="9" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E77" s="2" t="s">
         <v>10</v>
@@ -3264,7 +3268,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="78" spans="1:9">
       <c r="A78" s="8">
         <v>52014422850</v>
       </c>
@@ -3272,11 +3276,11 @@
         <v>2006</v>
       </c>
       <c r="C78" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A78,4)&amp;B78</f>
         <v>28502006</v>
       </c>
       <c r="D78" s="9" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E78" s="2" t="s">
         <v>10</v>
@@ -3294,7 +3298,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="79" spans="1:9">
       <c r="A79" s="8">
         <v>37446586869</v>
       </c>
@@ -3302,11 +3306,11 @@
         <v>1988</v>
       </c>
       <c r="C79" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A79,4)&amp;B79</f>
         <v>68691988</v>
       </c>
       <c r="D79" s="9" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E79" s="2" t="s">
         <v>10</v>
@@ -3324,7 +3328,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="80" spans="1:9">
       <c r="A80" s="8">
         <v>42672227896</v>
       </c>
@@ -3332,11 +3336,11 @@
         <v>1995</v>
       </c>
       <c r="C80" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A80,4)&amp;B80</f>
         <v>78961995</v>
       </c>
       <c r="D80" s="9" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="E80" s="2" t="s">
         <v>10</v>
@@ -3354,7 +3358,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="81" spans="1:9">
       <c r="A81" s="8">
         <v>51147754802</v>
       </c>
@@ -3362,11 +3366,11 @@
         <v>2001</v>
       </c>
       <c r="C81" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A81,4)&amp;B81</f>
         <v>48022001</v>
       </c>
       <c r="D81" s="9" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="E81" s="2" t="s">
         <v>10</v>
@@ -3384,7 +3388,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="82" spans="1:9">
       <c r="A82" s="10">
         <v>34606814896</v>
       </c>
@@ -3392,11 +3396,11 @@
         <v>1988</v>
       </c>
       <c r="C82" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A82,4)&amp;B82</f>
         <v>48961988</v>
       </c>
       <c r="D82" s="2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="E82" s="2" t="s">
         <v>10</v>
@@ -3414,7 +3418,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="83" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="83" spans="1:9">
       <c r="A83" s="8">
         <v>47211406810</v>
       </c>
@@ -3422,11 +3426,11 @@
         <v>2003</v>
       </c>
       <c r="C83" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A83,4)&amp;B83</f>
         <v>68102003</v>
       </c>
       <c r="D83" s="9" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E83" s="2" t="s">
         <v>10</v>
@@ -3444,19 +3448,19 @@
         <v>12</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="84" spans="1:9">
       <c r="A84" s="8">
-        <v>47817611866</v>
+        <v>42202090851</v>
       </c>
       <c r="B84" s="9">
         <v>1992</v>
       </c>
       <c r="C84" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v>18661992</v>
+        <f>RIGHT(A84,4)&amp;B84</f>
+        <v>08511992</v>
       </c>
       <c r="D84" s="9" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E84" s="2" t="s">
         <v>10</v>
@@ -3474,19 +3478,19 @@
         <v>12</v>
       </c>
     </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="85" spans="1:9">
       <c r="A85" s="8">
-        <v>42202090851</v>
+        <v>47817611866</v>
       </c>
       <c r="B85" s="9">
         <v>2000</v>
       </c>
       <c r="C85" s="2" t="str">
-        <f t="shared" si="2"/>
-        <v>08512000</v>
+        <f>RIGHT(A85,4)&amp;B85</f>
+        <v>18662000</v>
       </c>
       <c r="D85" s="9" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="E85" s="2" t="s">
         <v>10</v>
@@ -3504,7 +3508,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="86" spans="1:9">
       <c r="A86" s="8">
         <v>52353988822</v>
       </c>
@@ -3512,11 +3516,11 @@
         <v>2003</v>
       </c>
       <c r="C86" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A86,4)&amp;B86</f>
         <v>88222003</v>
       </c>
       <c r="D86" s="9" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="E86" s="2" t="s">
         <v>10</v>
@@ -3534,7 +3538,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="87" spans="1:9">
       <c r="A87" s="8">
         <v>44350770860</v>
       </c>
@@ -3542,11 +3546,11 @@
         <v>2002</v>
       </c>
       <c r="C87" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A87,4)&amp;B87</f>
         <v>08602002</v>
       </c>
       <c r="D87" s="9" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="E87" s="2" t="s">
         <v>10</v>
@@ -3564,7 +3568,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="88" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="88" spans="1:9">
       <c r="A88" s="8">
         <v>38011287842</v>
       </c>
@@ -3572,11 +3576,11 @@
         <v>2001</v>
       </c>
       <c r="C88" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A88,4)&amp;B88</f>
         <v>78422001</v>
       </c>
       <c r="D88" s="9" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="E88" s="2" t="s">
         <v>10</v>
@@ -3594,7 +3598,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="89" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="89" spans="1:9">
       <c r="A89" s="8">
         <v>8817038342</v>
       </c>
@@ -3602,11 +3606,11 @@
         <v>2004</v>
       </c>
       <c r="C89" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A89,4)&amp;B89</f>
         <v>83422004</v>
       </c>
       <c r="D89" s="9" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="E89" s="2" t="s">
         <v>10</v>
@@ -3624,7 +3628,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="90" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="90" spans="1:9">
       <c r="A90" s="8">
         <v>770030475</v>
       </c>
@@ -3632,11 +3636,11 @@
         <v>1979</v>
       </c>
       <c r="C90" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A90,4)&amp;B90</f>
         <v>04751979</v>
       </c>
       <c r="D90" s="9" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="E90" s="2" t="s">
         <v>10</v>
@@ -3654,7 +3658,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="91" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="91" spans="1:9">
       <c r="A91" s="8">
         <v>45989936850</v>
       </c>
@@ -3662,11 +3666,11 @@
         <v>1997</v>
       </c>
       <c r="C91" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A91,4)&amp;B91</f>
         <v>68501997</v>
       </c>
       <c r="D91" s="9" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="E91" s="2" t="s">
         <v>10</v>
@@ -3684,7 +3688,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="92" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="92" spans="1:9">
       <c r="A92" s="8">
         <v>41460506855</v>
       </c>
@@ -3692,11 +3696,11 @@
         <v>2005</v>
       </c>
       <c r="C92" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A92,4)&amp;B92</f>
         <v>68552005</v>
       </c>
       <c r="D92" s="9" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="E92" s="2" t="s">
         <v>10</v>
@@ -3714,7 +3718,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="93" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="93" spans="1:9">
       <c r="A93" s="8">
         <v>47167140805</v>
       </c>
@@ -3722,11 +3726,11 @@
         <v>2000</v>
       </c>
       <c r="C93" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A93,4)&amp;B93</f>
         <v>08052000</v>
       </c>
       <c r="D93" s="9" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="E93" s="2" t="s">
         <v>10</v>
@@ -3744,7 +3748,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="94" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="94" spans="1:9">
       <c r="A94" s="8">
         <v>32568233869</v>
       </c>
@@ -3752,11 +3756,11 @@
         <v>1985</v>
       </c>
       <c r="C94" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A94,4)&amp;B94</f>
         <v>38691985</v>
       </c>
       <c r="D94" s="9" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="E94" s="2" t="s">
         <v>10</v>
@@ -3774,7 +3778,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="95" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="95" spans="1:9">
       <c r="A95" s="8">
         <v>53833326859</v>
       </c>
@@ -3782,11 +3786,11 @@
         <v>2006</v>
       </c>
       <c r="C95" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A95,4)&amp;B95</f>
         <v>68592006</v>
       </c>
       <c r="D95" s="9" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="E95" s="2" t="s">
         <v>10</v>
@@ -3804,7 +3808,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="96" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="96" spans="1:9">
       <c r="A96" s="8">
         <v>52172623890</v>
       </c>
@@ -3812,11 +3816,11 @@
         <v>2005</v>
       </c>
       <c r="C96" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A96,4)&amp;B96</f>
         <v>38902005</v>
       </c>
       <c r="D96" s="9" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="E96" s="2" t="s">
         <v>10</v>
@@ -3834,7 +3838,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="97" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="97" spans="1:9">
       <c r="A97" s="8">
         <v>34884914805</v>
       </c>
@@ -3842,11 +3846,11 @@
         <v>1985</v>
       </c>
       <c r="C97" s="2" t="str">
-        <f t="shared" si="2"/>
+        <f>RIGHT(A97,4)&amp;B97</f>
         <v>48051985</v>
       </c>
       <c r="D97" s="9" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="E97" s="2" t="s">
         <v>10</v>
@@ -3864,7 +3868,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="98" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="98" spans="1:9">
       <c r="A98" s="8">
         <v>41755663846</v>
       </c>
@@ -3872,11 +3876,11 @@
         <v>2002</v>
       </c>
       <c r="C98" s="2" t="str">
-        <f t="shared" ref="C98:C129" si="3">RIGHT(A98,4)&amp;B98</f>
+        <f>RIGHT(A98,4)&amp;B98</f>
         <v>38462002</v>
       </c>
       <c r="D98" s="9" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="E98" s="2" t="s">
         <v>10</v>
@@ -3894,7 +3898,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="99" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="99" spans="1:9">
       <c r="A99" s="8">
         <v>42222464846</v>
       </c>
@@ -3902,11 +3906,11 @@
         <v>1994</v>
       </c>
       <c r="C99" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A99,4)&amp;B99</f>
         <v>48461994</v>
       </c>
       <c r="D99" s="9" t="s">
-        <v>113</v>
+        <v>114</v>
       </c>
       <c r="E99" s="2" t="s">
         <v>10</v>
@@ -3924,7 +3928,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="100" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="100" spans="1:9">
       <c r="A100" s="8">
         <v>57536852851</v>
       </c>
@@ -3932,11 +3936,11 @@
         <v>2008</v>
       </c>
       <c r="C100" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A100,4)&amp;B100</f>
         <v>28512008</v>
       </c>
       <c r="D100" s="9" t="s">
-        <v>114</v>
+        <v>115</v>
       </c>
       <c r="E100" s="2" t="s">
         <v>10</v>
@@ -3954,7 +3958,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="101" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="101" spans="1:9">
       <c r="A101" s="8">
         <v>48556621864</v>
       </c>
@@ -3962,11 +3966,11 @@
         <v>2000</v>
       </c>
       <c r="C101" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A101,4)&amp;B101</f>
         <v>18642000</v>
       </c>
       <c r="D101" s="9" t="s">
-        <v>115</v>
+        <v>116</v>
       </c>
       <c r="E101" s="2" t="s">
         <v>10</v>
@@ -3984,7 +3988,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="102" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="102" spans="1:9">
       <c r="A102" s="8">
         <v>50308043820</v>
       </c>
@@ -3992,11 +3996,11 @@
         <v>2001</v>
       </c>
       <c r="C102" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A102,4)&amp;B102</f>
         <v>38202001</v>
       </c>
       <c r="D102" s="9" t="s">
-        <v>116</v>
+        <v>117</v>
       </c>
       <c r="E102" s="2" t="s">
         <v>10</v>
@@ -4014,7 +4018,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="103" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="103" spans="1:9">
       <c r="A103" s="8">
         <v>45279130850</v>
       </c>
@@ -4022,11 +4026,11 @@
         <v>2003</v>
       </c>
       <c r="C103" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A103,4)&amp;B103</f>
         <v>08502003</v>
       </c>
       <c r="D103" s="9" t="s">
-        <v>117</v>
+        <v>118</v>
       </c>
       <c r="E103" s="2" t="s">
         <v>10</v>
@@ -4044,7 +4048,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="104" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="104" spans="1:9">
       <c r="A104" s="8">
         <v>49190532821</v>
       </c>
@@ -4052,11 +4056,11 @@
         <v>2003</v>
       </c>
       <c r="C104" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A104,4)&amp;B104</f>
         <v>28212003</v>
       </c>
       <c r="D104" s="9" t="s">
-        <v>118</v>
+        <v>119</v>
       </c>
       <c r="E104" s="2" t="s">
         <v>10</v>
@@ -4074,7 +4078,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="105" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="105" spans="1:9">
       <c r="A105" s="8">
         <v>53864652871</v>
       </c>
@@ -4082,11 +4086,11 @@
         <v>2006</v>
       </c>
       <c r="C105" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A105,4)&amp;B105</f>
         <v>28712006</v>
       </c>
       <c r="D105" s="9" t="s">
-        <v>119</v>
+        <v>120</v>
       </c>
       <c r="E105" s="2" t="s">
         <v>10</v>
@@ -4104,7 +4108,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="106" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="106" spans="1:9">
       <c r="A106" s="8">
         <v>52587009847</v>
       </c>
@@ -4112,11 +4116,11 @@
         <v>2004</v>
       </c>
       <c r="C106" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A106,4)&amp;B106</f>
         <v>98472004</v>
       </c>
       <c r="D106" s="9" t="s">
-        <v>120</v>
+        <v>121</v>
       </c>
       <c r="E106" s="2" t="s">
         <v>10</v>
@@ -4134,7 +4138,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="107" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="107" spans="1:9">
       <c r="A107" s="8">
         <v>29911349845</v>
       </c>
@@ -4142,11 +4146,11 @@
         <v>1981</v>
       </c>
       <c r="C107" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A107,4)&amp;B107</f>
         <v>98451981</v>
       </c>
       <c r="D107" s="9" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E107" s="2" t="s">
         <v>10</v>
@@ -4164,7 +4168,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="108" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="108" spans="1:9">
       <c r="A108" s="8">
         <v>52970856832</v>
       </c>
@@ -4172,11 +4176,11 @@
         <v>2001</v>
       </c>
       <c r="C108" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A108,4)&amp;B108</f>
         <v>68322001</v>
       </c>
       <c r="D108" s="9" t="s">
-        <v>122</v>
+        <v>123</v>
       </c>
       <c r="E108" s="2" t="s">
         <v>10</v>
@@ -4194,7 +4198,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="109" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="109" spans="1:9">
       <c r="A109" s="8">
         <v>33020819873</v>
       </c>
@@ -4202,11 +4206,11 @@
         <v>1985</v>
       </c>
       <c r="C109" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A109,4)&amp;B109</f>
         <v>98731985</v>
       </c>
       <c r="D109" s="9" t="s">
-        <v>123</v>
+        <v>124</v>
       </c>
       <c r="E109" s="2" t="s">
         <v>10</v>
@@ -4224,7 +4228,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="110" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="110" spans="1:9">
       <c r="A110" s="8">
         <v>33091270874</v>
       </c>
@@ -4232,11 +4236,11 @@
         <v>1986</v>
       </c>
       <c r="C110" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A110,4)&amp;B110</f>
         <v>08741986</v>
       </c>
       <c r="D110" s="9" t="s">
-        <v>124</v>
+        <v>125</v>
       </c>
       <c r="E110" s="2" t="s">
         <v>10</v>
@@ -4254,7 +4258,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="111" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="111" spans="1:9">
       <c r="A111" s="8">
         <v>27378843814</v>
       </c>
@@ -4262,11 +4266,11 @@
         <v>1977</v>
       </c>
       <c r="C111" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A111,4)&amp;B111</f>
         <v>38141977</v>
       </c>
       <c r="D111" s="9" t="s">
-        <v>125</v>
+        <v>126</v>
       </c>
       <c r="E111" s="2" t="s">
         <v>10</v>
@@ -4284,7 +4288,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="112" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="112" spans="1:9">
       <c r="A112" s="8">
         <v>40165009829</v>
       </c>
@@ -4292,11 +4296,11 @@
         <v>2007</v>
       </c>
       <c r="C112" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A112,4)&amp;B112</f>
         <v>98292007</v>
       </c>
       <c r="D112" s="9" t="s">
-        <v>126</v>
+        <v>127</v>
       </c>
       <c r="E112" s="2" t="s">
         <v>10</v>
@@ -4314,7 +4318,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="113" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="113" spans="1:9">
       <c r="A113" s="8">
         <v>29170771820</v>
       </c>
@@ -4322,11 +4326,11 @@
         <v>1982</v>
       </c>
       <c r="C113" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A113,4)&amp;B113</f>
         <v>18201982</v>
       </c>
       <c r="D113" s="9" t="s">
-        <v>127</v>
+        <v>128</v>
       </c>
       <c r="E113" s="2" t="s">
         <v>10</v>
@@ -4344,7 +4348,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="114" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="114" spans="1:9">
       <c r="A114" s="8">
         <v>25516190843</v>
       </c>
@@ -4352,11 +4356,11 @@
         <v>1975</v>
       </c>
       <c r="C114" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A114,4)&amp;B114</f>
         <v>08431975</v>
       </c>
       <c r="D114" s="9" t="s">
-        <v>128</v>
+        <v>129</v>
       </c>
       <c r="E114" s="2" t="s">
         <v>10</v>
@@ -4374,7 +4378,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="115" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="115" spans="1:9">
       <c r="A115" s="8">
         <v>26192473811</v>
       </c>
@@ -4382,11 +4386,11 @@
         <v>1977</v>
       </c>
       <c r="C115" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A115,4)&amp;B115</f>
         <v>38111977</v>
       </c>
       <c r="D115" s="9" t="s">
-        <v>129</v>
+        <v>130</v>
       </c>
       <c r="E115" s="2" t="s">
         <v>10</v>
@@ -4404,7 +4408,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="116" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="116" spans="1:9">
       <c r="A116" s="8">
         <v>36322128809</v>
       </c>
@@ -4412,11 +4416,11 @@
         <v>1990</v>
       </c>
       <c r="C116" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A116,4)&amp;B116</f>
         <v>88091990</v>
       </c>
       <c r="D116" s="9" t="s">
-        <v>130</v>
+        <v>131</v>
       </c>
       <c r="E116" s="2" t="s">
         <v>10</v>
@@ -4434,7 +4438,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="117" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="117" spans="1:9">
       <c r="A117" s="8">
         <v>28469113801</v>
       </c>
@@ -4442,11 +4446,11 @@
         <v>1980</v>
       </c>
       <c r="C117" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A117,4)&amp;B117</f>
         <v>38011980</v>
       </c>
       <c r="D117" s="9" t="s">
-        <v>131</v>
+        <v>132</v>
       </c>
       <c r="E117" s="2" t="s">
         <v>10</v>
@@ -4464,7 +4468,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="118" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="118" spans="1:9">
       <c r="A118" s="8">
         <v>31014693845</v>
       </c>
@@ -4472,11 +4476,11 @@
         <v>1984</v>
       </c>
       <c r="C118" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A118,4)&amp;B118</f>
         <v>38451984</v>
       </c>
       <c r="D118" s="9" t="s">
-        <v>132</v>
+        <v>133</v>
       </c>
       <c r="E118" s="2" t="s">
         <v>10</v>
@@ -4494,7 +4498,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="119" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="119" spans="1:9">
       <c r="A119" s="8">
         <v>33887811844</v>
       </c>
@@ -4502,11 +4506,11 @@
         <v>1984</v>
       </c>
       <c r="C119" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A119,4)&amp;B119</f>
         <v>18441984</v>
       </c>
       <c r="D119" s="9" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E119" s="2" t="s">
         <v>10</v>
@@ -4524,7 +4528,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="120" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="120" spans="1:9">
       <c r="A120" s="8">
         <v>28505783808</v>
       </c>
@@ -4532,11 +4536,11 @@
         <v>1980</v>
       </c>
       <c r="C120" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A120,4)&amp;B120</f>
         <v>38081980</v>
       </c>
       <c r="D120" s="9" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="E120" s="2" t="s">
         <v>10</v>
@@ -4554,19 +4558,19 @@
         <v>12</v>
       </c>
     </row>
-    <row r="121" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="121" spans="1:9">
       <c r="A121" s="1" t="s">
-        <v>135</v>
+        <v>136</v>
       </c>
       <c r="B121" s="2">
         <v>1960</v>
       </c>
       <c r="C121" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A121,4)&amp;B121</f>
         <v>78051960</v>
       </c>
       <c r="D121" s="2" t="s">
-        <v>136</v>
+        <v>137</v>
       </c>
       <c r="E121" s="2" t="s">
         <v>10</v>
@@ -4584,7 +4588,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="122" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="122" spans="1:9">
       <c r="A122" s="8">
         <v>48060547801</v>
       </c>
@@ -4592,11 +4596,11 @@
         <v>1997</v>
       </c>
       <c r="C122" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A122,4)&amp;B122</f>
         <v>78011997</v>
       </c>
       <c r="D122" s="9" t="s">
-        <v>137</v>
+        <v>138</v>
       </c>
       <c r="E122" s="2" t="s">
         <v>10</v>
@@ -4614,7 +4618,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="123" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="123" spans="1:9">
       <c r="A123" s="8">
         <v>26687173880</v>
       </c>
@@ -4622,11 +4626,11 @@
         <v>1975</v>
       </c>
       <c r="C123" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A123,4)&amp;B123</f>
         <v>38801975</v>
       </c>
       <c r="D123" s="9" t="s">
-        <v>138</v>
+        <v>139</v>
       </c>
       <c r="E123" s="2" t="s">
         <v>10</v>
@@ -4644,7 +4648,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="124" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="124" spans="1:9">
       <c r="A124" s="8">
         <v>44610167816</v>
       </c>
@@ -4652,11 +4656,11 @@
         <v>1995</v>
       </c>
       <c r="C124" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A124,4)&amp;B124</f>
         <v>78161995</v>
       </c>
       <c r="D124" s="9" t="s">
-        <v>139</v>
+        <v>140</v>
       </c>
       <c r="E124" s="2" t="s">
         <v>10</v>
@@ -4674,7 +4678,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="125" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="125" spans="1:9">
       <c r="A125" s="8">
         <v>37196678800</v>
       </c>
@@ -4682,11 +4686,11 @@
         <v>1989</v>
       </c>
       <c r="C125" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A125,4)&amp;B125</f>
         <v>88001989</v>
       </c>
       <c r="D125" s="9" t="s">
-        <v>140</v>
+        <v>141</v>
       </c>
       <c r="E125" s="2" t="s">
         <v>10</v>
@@ -4704,7 +4708,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="126" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="126" spans="1:9">
       <c r="A126" s="8">
         <v>34294701889</v>
       </c>
@@ -4712,11 +4716,11 @@
         <v>1986</v>
       </c>
       <c r="C126" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A126,4)&amp;B126</f>
         <v>18891986</v>
       </c>
       <c r="D126" s="9" t="s">
-        <v>141</v>
+        <v>142</v>
       </c>
       <c r="E126" s="2" t="s">
         <v>10</v>
@@ -4734,7 +4738,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="127" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="127" spans="1:9">
       <c r="A127" s="8">
         <v>50400969840</v>
       </c>
@@ -4742,11 +4746,11 @@
         <v>2002</v>
       </c>
       <c r="C127" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A127,4)&amp;B127</f>
         <v>98402002</v>
       </c>
       <c r="D127" s="9" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="E127" s="2" t="s">
         <v>10</v>
@@ -4764,7 +4768,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="128" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="128" spans="1:9">
       <c r="A128" s="8">
         <v>39724385833</v>
       </c>
@@ -4772,11 +4776,11 @@
         <v>1991</v>
       </c>
       <c r="C128" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A128,4)&amp;B128</f>
         <v>58331991</v>
       </c>
       <c r="D128" s="9" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="E128" s="2" t="s">
         <v>10</v>
@@ -4794,7 +4798,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="129" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="129" spans="1:9">
       <c r="A129" s="8">
         <v>20053874870</v>
       </c>
@@ -4802,11 +4806,11 @@
         <v>1976</v>
       </c>
       <c r="C129" s="2" t="str">
-        <f t="shared" si="3"/>
+        <f>RIGHT(A129,4)&amp;B129</f>
         <v>48701976</v>
       </c>
       <c r="D129" s="9" t="s">
-        <v>144</v>
+        <v>145</v>
       </c>
       <c r="E129" s="2" t="s">
         <v>10</v>
@@ -4824,7 +4828,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="130" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="130" spans="1:9">
       <c r="A130" s="15">
         <v>40542592860</v>
       </c>
@@ -4832,13 +4836,13 @@
         <v>1992</v>
       </c>
       <c r="C130" s="12" t="str">
-        <f t="shared" ref="C130:C161" si="4">RIGHT(A130,4)&amp;B130</f>
+        <f>RIGHT(A130,4)&amp;B130</f>
         <v>28601992</v>
       </c>
       <c r="D130" s="16" t="s">
-        <v>145</v>
-      </c>
-      <c r="E130" s="12" t="s">
+        <v>146</v>
+      </c>
+      <c r="E130" s="2" t="s">
         <v>10</v>
       </c>
       <c r="F130" s="12">
@@ -4854,7 +4858,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="131" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="131" spans="1:9">
       <c r="A131" s="8">
         <v>48963889840</v>
       </c>
@@ -4862,11 +4866,11 @@
         <v>2000</v>
       </c>
       <c r="C131" s="2" t="str">
-        <f t="shared" si="4"/>
+        <f>RIGHT(A131,4)&amp;B131</f>
         <v>98402000</v>
       </c>
       <c r="D131" s="9" t="s">
-        <v>146</v>
+        <v>147</v>
       </c>
       <c r="E131" s="2" t="s">
         <v>10</v>
@@ -4884,7 +4888,7 @@
         <v>12</v>
       </c>
     </row>
-    <row r="132" spans="1:9" x14ac:dyDescent="0.35">
+    <row r="132" spans="1:9">
       <c r="A132" s="8">
         <v>44273964880</v>
       </c>
@@ -4892,11 +4896,11 @@
         <v>1993</v>
       </c>
       <c r="C132" s="2" t="str">
-        <f t="shared" si="4"/>
+        <f>RIGHT(A132,4)&amp;B132</f>
         <v>48801993</v>
       </c>
       <c r="D132" s="9" t="s">
-        <v>147</v>
+        <v>148</v>
       </c>
       <c r="E132" s="2" t="s">
         <v>10</v>
@@ -4915,6 +4919,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection algorithmName="SHA-512" hashValue="JAmitZ7/9q7yf5sGrdgz940vCRy6HkorJ/kbDEI3TDZsoJlmiE+IJQDnQZsokuX8469elukOQx8MMceph+f8ew==" saltValue="6hclAJOWB9mV9SkIlXGe0g==" spinCount="100000" sheet="1" objects="1" scenarios="1" selectLockedCells="1" selectUnlockedCells="1"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>